<commit_message>
Haftalik veri guncellemesi (2026-07-31)
python haftalik_calistir.py ile 21/21 adim basarili: fon performansi,
F/K ucluesu, peer F/K, BIST yillik getiriler, endeks serileri ve 13
fonun fiyat grafigi guncellendi.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1466,7 +1466,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>13944</v>
+        <v>13775</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>13000</v>
@@ -1490,7 +1490,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1514,7 +1514,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1538,7 +1538,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1562,7 +1562,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>6281</v>
+        <v>6282</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>5800</v>
@@ -4393,7 +4393,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B2" s="8" t="n">
@@ -5177,7 +5177,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>16.4</v>
+        <v>15.7</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5231,7 +5231,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>40.8</v>
+        <v>38.9</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5249,7 +5249,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>28.5</v>
+        <v>27.1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5267,7 +5267,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>30.2</v>
+        <v>28.6</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5303,7 +5303,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>50.5</v>
+        <v>50.2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5321,7 +5321,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>46.3</v>
+        <v>45.9</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5339,7 +5339,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>47.4</v>
+        <v>47.1</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5357,7 +5357,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>36.8</v>
+        <v>38</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5375,7 +5375,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>47.2</v>
+        <v>52.5</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5393,7 +5393,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>23.5</v>
+        <v>22.7</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5411,7 +5411,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>28.2</v>
+        <v>45.6</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5429,7 +5429,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>36.7</v>
+        <v>38.9</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5447,7 +5447,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>31.6</v>
+        <v>32.7</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5580,7 +5580,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>14.3</v>
+        <v>13.4</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12.6</v>
+        <v>12.1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5616,7 +5616,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>30.9</v>
+        <v>29.7</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5634,7 +5634,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>11.1</v>
+        <v>25.5</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5652,7 +5652,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>15.6</v>
+        <v>14.2</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5670,7 +5670,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>28.2</v>
+        <v>27.6</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5688,7 +5688,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>27</v>
+        <v>31.4</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5706,7 +5706,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>21.3</v>
+        <v>19.4</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5724,7 +5724,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>24.3</v>
+        <v>22.3</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5742,7 +5742,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>22.4</v>
+        <v>21.9</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5760,7 +5760,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>23.9</v>
+        <v>24</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5778,7 +5778,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-1.8</v>
+        <v>-1</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5796,7 +5796,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5814,7 +5814,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5832,7 +5832,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>13.3</v>
+        <v>14.4</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5850,7 +5850,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.4</v>
+        <v>10.5</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5868,7 +5868,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>25.5</v>
+        <v>25.6</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>22.3</v>
+        <v>22.4</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -6855,7 +6855,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6869,16 +6869,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="E2" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6892,16 +6892,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>10.1</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6918,13 +6918,13 @@
         <v>19.2</v>
       </c>
       <c r="E4" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6938,16 +6938,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>46.3</v>
+        <v>45.9</v>
       </c>
       <c r="E5" t="n">
-        <v>45.9</v>
+        <v>45.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6961,16 +6961,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>22.3</v>
+        <v>22.4</v>
       </c>
       <c r="E6" t="n">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6984,16 +6984,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.9</v>
+        <v>-0.6</v>
       </c>
       <c r="E7" t="n">
-        <v>-4.8</v>
+        <v>-7.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -7007,16 +7007,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>-3.2</v>
+        <v>-2.1</v>
       </c>
       <c r="E8" t="n">
-        <v>-7.3</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -7030,16 +7030,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>4.9</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>5.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -7056,13 +7056,13 @@
         <v>29.7</v>
       </c>
       <c r="E10" t="n">
-        <v>28.5</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -7076,16 +7076,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>22.4</v>
+        <v>21.9</v>
       </c>
       <c r="E11" t="n">
-        <v>21.3</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -7099,16 +7099,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>5.9</v>
+        <v>5.2</v>
       </c>
       <c r="E12" t="n">
-        <v>6.2</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -7122,7 +7122,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="E13" t="n">
         <v>6.6</v>
@@ -7131,7 +7131,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7145,16 +7145,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>17.8</v>
+        <v>15.5</v>
       </c>
       <c r="E14" t="n">
-        <v>18.9</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -7168,16 +7168,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>36.8</v>
+        <v>38</v>
       </c>
       <c r="E15" t="n">
-        <v>41.8</v>
+        <v>42.6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7191,7 +7191,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>28.2</v>
+        <v>27.6</v>
       </c>
       <c r="E16" t="n">
         <v>32.3</v>
@@ -7200,7 +7200,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -7214,16 +7214,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>-11</v>
+        <v>-10.7</v>
       </c>
       <c r="E17" t="n">
-        <v>1.9</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7237,16 +7237,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E18" t="n">
-        <v>20.1</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7260,16 +7260,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>31.3</v>
+        <v>27.3</v>
       </c>
       <c r="E19" t="n">
-        <v>36.9</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7283,16 +7283,16 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>47.2</v>
+        <v>52.5</v>
       </c>
       <c r="E20" t="n">
-        <v>50.5</v>
+        <v>48.9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7306,16 +7306,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>27</v>
+        <v>31.4</v>
       </c>
       <c r="E21" t="n">
-        <v>46.7</v>
+        <v>44.5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7329,16 +7329,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1.7</v>
+        <v>-2.2</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7352,16 +7352,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="E23" t="n">
-        <v>11.8</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7375,16 +7375,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3.1</v>
+        <v>1.2</v>
       </c>
       <c r="E24" t="n">
-        <v>19.1</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7398,16 +7398,16 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>23.5</v>
+        <v>22.7</v>
       </c>
       <c r="E25" t="n">
-        <v>39</v>
+        <v>37.2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7421,16 +7421,16 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>15.6</v>
+        <v>14.2</v>
       </c>
       <c r="E26" t="n">
-        <v>33.1</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7444,16 +7444,16 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>-5.5</v>
+        <v>5.1</v>
       </c>
       <c r="E27" t="n">
-        <v>-8.300000000000001</v>
+        <v>-6.7</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7467,16 +7467,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>-15.3</v>
+        <v>-2.3</v>
       </c>
       <c r="E28" t="n">
-        <v>-20.9</v>
+        <v>-17.4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7490,16 +7490,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>-11</v>
+        <v>-0.4</v>
       </c>
       <c r="E29" t="n">
-        <v>-12.7</v>
+        <v>-10.8</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7513,16 +7513,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>28.2</v>
+        <v>45.6</v>
       </c>
       <c r="E30" t="n">
-        <v>20.1</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7536,16 +7536,16 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>11.1</v>
+        <v>25.5</v>
       </c>
       <c r="E31" t="n">
-        <v>5.2</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7559,16 +7559,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>-1.3</v>
+        <v>-0.7</v>
       </c>
       <c r="E32" t="n">
-        <v>0.5</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7582,16 +7582,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>-5.4</v>
+        <v>-4.3</v>
       </c>
       <c r="E33" t="n">
-        <v>-2</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7605,16 +7605,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.1</v>
+        <v>-1.7</v>
       </c>
       <c r="E34" t="n">
-        <v>7.9</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7631,13 +7631,13 @@
         <v>19.5</v>
       </c>
       <c r="E35" t="n">
-        <v>30.2</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7651,16 +7651,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>12.6</v>
+        <v>12.1</v>
       </c>
       <c r="E36" t="n">
-        <v>24.3</v>
+        <v>22.3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7674,16 +7674,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4511.5</v>
+        <v>4491.6</v>
       </c>
       <c r="E37" t="n">
-        <v>4946.1</v>
+        <v>4865.8</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7697,16 +7697,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>-2.3</v>
+        <v>-3.4</v>
       </c>
       <c r="E38" t="n">
-        <v>-4.8</v>
+        <v>-7.4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7720,16 +7720,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>-5.2</v>
+        <v>-4.5</v>
       </c>
       <c r="E39" t="n">
-        <v>-7.3</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7743,16 +7743,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>-1.8</v>
       </c>
       <c r="E40" t="n">
-        <v>5.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7766,16 +7766,16 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>16.4</v>
+        <v>15.7</v>
       </c>
       <c r="E41" t="n">
-        <v>28.5</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7789,16 +7789,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>14.3</v>
+        <v>13.4</v>
       </c>
       <c r="E42" t="n">
-        <v>21.3</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7812,16 +7812,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>5843.8</v>
+        <v>5798.5</v>
       </c>
       <c r="E43" t="n">
-        <v>2605.6</v>
+        <v>2563.8</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7835,16 +7835,16 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>121.3</v>
+        <v>115.1</v>
       </c>
       <c r="E44" t="n">
-        <v>103.6</v>
+        <v>96.3</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7858,16 +7858,16 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1223.5</v>
+        <v>1213.4</v>
       </c>
       <c r="E45" t="n">
-        <v>995.5</v>
+        <v>978.5</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7881,16 +7881,16 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2.6</v>
+        <v>0.5</v>
       </c>
       <c r="E46" t="n">
-        <v>4.1</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7904,16 +7904,16 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>4.5</v>
+        <v>5.1</v>
       </c>
       <c r="E47" t="n">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7927,16 +7927,16 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>14.3</v>
+        <v>11.3</v>
       </c>
       <c r="E48" t="n">
-        <v>22.7</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7950,16 +7950,16 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>40.8</v>
+        <v>38.9</v>
       </c>
       <c r="E49" t="n">
-        <v>51.1</v>
+        <v>48.7</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7973,16 +7973,16 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>30.9</v>
+        <v>29.7</v>
       </c>
       <c r="E50" t="n">
-        <v>40.6</v>
+        <v>38.9</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -7996,16 +7996,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.4</v>
+        <v>3.1</v>
       </c>
       <c r="E51" t="n">
-        <v>1.2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -8019,16 +8019,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>-9.9</v>
+        <v>-7.8</v>
       </c>
       <c r="E52" t="n">
-        <v>-7.8</v>
+        <v>-6.2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -8042,16 +8042,16 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-11.8</v>
+        <v>-13.9</v>
       </c>
       <c r="E53" t="n">
-        <v>-8.4</v>
+        <v>-10.3</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -8065,16 +8065,16 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>36.7</v>
+        <v>38.9</v>
       </c>
       <c r="E54" t="n">
-        <v>40.4</v>
+        <v>41.7</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -8088,7 +8088,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>-1.8</v>
+        <v>-1</v>
       </c>
       <c r="E55" t="n">
         <v>2.4</v>
@@ -8097,7 +8097,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -8111,13 +8111,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>-0.4</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -8131,13 +8131,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>3.6</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -8151,13 +8151,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>11.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -8171,13 +8171,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>31.6</v>
+        <v>32.7</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -8191,13 +8191,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>13.3</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -8211,16 +8211,16 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="E61" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -8243,7 +8243,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -8266,7 +8266,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -8280,16 +8280,16 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>50.5</v>
+        <v>50.2</v>
       </c>
       <c r="E64" t="n">
-        <v>47.4</v>
+        <v>47.1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -8303,16 +8303,16 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>25.5</v>
+        <v>25.6</v>
       </c>
       <c r="E65" t="n">
-        <v>23.9</v>
+        <v>24</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -8335,7 +8335,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -8349,7 +8349,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
       <c r="E67" t="n">
         <v>0.6</v>
@@ -8358,7 +8358,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -8372,7 +8372,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>9.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E68" t="n">
         <v>1.1</v>
@@ -8381,7 +8381,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -8404,7 +8404,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -8418,7 +8418,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="E70" t="n">
         <v>1.2</v>
@@ -8427,7 +8427,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -8441,13 +8441,13 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -8467,7 +8467,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -8544,7 +8544,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8569,7 +8569,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8588,13 +8588,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8613,13 +8613,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>9.5</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8644,7 +8644,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8663,13 +8663,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>10.4</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8688,13 +8688,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8719,7 +8719,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8744,7 +8744,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8763,13 +8763,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>47.4</v>
+        <v>47.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -8788,13 +8788,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>23.9</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -8813,13 +8813,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>7.4</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -8838,13 +8838,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -8863,13 +8863,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>16.7</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -8888,13 +8888,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>36.1</v>
+        <v>37.1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -8913,13 +8913,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>27.9</v>
+        <v>28.3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -8938,13 +8938,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -8963,13 +8963,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>11.8</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -8988,13 +8988,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>23.1</v>
+        <v>20.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9013,13 +9013,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>52.5</v>
+        <v>52.8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9038,13 +9038,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>40.5</v>
+        <v>39.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9063,13 +9063,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>-1.2</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9088,13 +9088,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>9.5</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9113,13 +9113,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9138,13 +9138,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>23.6</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9163,13 +9163,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>14.3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -9188,13 +9188,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>7.5</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -9213,13 +9213,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>39.8</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -9238,13 +9238,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>88.90000000000001</v>
+        <v>78.09999999999999</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -9263,13 +9263,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>100.4</v>
+        <v>93.3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -9288,13 +9288,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>106.8</v>
+        <v>97.40000000000001</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -9319,7 +9319,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -9338,13 +9338,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>10.8</v>
+        <v>10.79</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -9363,13 +9363,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>22.2</v>
+        <v>22.21</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -9388,13 +9388,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>50.6</v>
+        <v>50.57</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -9413,7 +9413,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>25.87</v>
+        <v>26.01</v>
       </c>
     </row>
   </sheetData>
@@ -9527,7 +9527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9561,7 +9561,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9575,13 +9575,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>15.13</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9595,13 +9595,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>13.99</v>
+        <v>14.52</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9615,13 +9615,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.2</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9635,13 +9635,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2.47</v>
+        <v>2.57</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9655,13 +9655,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4.45</v>
+        <v>4.62</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9675,13 +9675,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>37.89</v>
+        <v>36.95</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9695,13 +9695,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5.46</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9715,13 +9715,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>19.41</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -9735,13 +9735,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5.67</v>
+        <v>5.63</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -9755,13 +9755,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>77.45</v>
+        <v>77.39</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>16.88</v>
+        <v>16.98</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -9795,13 +9795,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>83.93000000000001</v>
+        <v>83.14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -9815,13 +9815,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>12.56</v>
+        <v>13.32</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -9835,13 +9835,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3.51</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -9861,7 +9861,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9875,13 +9875,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3.57</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -9895,13 +9895,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>66.01000000000001</v>
+        <v>65.08</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -9915,13 +9915,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1.13</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9935,13 +9935,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.7</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9955,13 +9955,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>13.99</v>
+        <v>15.31</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9975,13 +9975,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>13.09</v>
+        <v>12.76</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9991,17 +9991,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Kamu Dış Borçlanma Araçları</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>96.88</v>
+        <v>3.12</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -10011,17 +10011,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Özel Sektör Dış Borçlanma Araçları</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3.12</v>
+        <v>96.88</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -10035,13 +10035,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>81</v>
+        <v>81.31</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -10061,7 +10061,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -10075,13 +10075,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>4.08</v>
+        <v>3.79</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -10095,13 +10095,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2.84</v>
+        <v>2.88</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -10115,13 +10115,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>11.16</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -10135,13 +10135,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1.57</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -10161,7 +10161,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -10175,13 +10175,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>41.22</v>
+        <v>38.28</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -10201,7 +10201,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -10215,13 +10215,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>55.06</v>
+        <v>57.99</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>22.71</v>
+        <v>22.01</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -10255,13 +10255,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.2</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -10275,13 +10275,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>71.38</v>
+        <v>70.58</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -10295,13 +10295,13 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>5.71</v>
+        <v>5.59</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -10315,13 +10315,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>3.44</v>
+        <v>3.41</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -10335,13 +10335,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>94.70999999999999</v>
+        <v>94.84999999999999</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -10355,13 +10355,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1.85</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -10375,13 +10375,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>72.05</v>
+        <v>72.13</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -10395,13 +10395,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27.95</v>
+        <v>27.87</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -10415,13 +10415,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>22.05</v>
+        <v>20.76</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -10435,13 +10435,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.22</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10455,13 +10455,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>64.84</v>
+        <v>66.09</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -10475,13 +10475,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>12.89</v>
+        <v>12.33</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -10495,13 +10495,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>92.15000000000001</v>
+        <v>90.31</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -10515,13 +10515,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>7.85</v>
+        <v>9.69</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -10535,13 +10535,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.62</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -10555,13 +10555,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>15.14</v>
+        <v>14.88</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -10571,17 +10571,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>1.62</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -10591,17 +10591,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.09</v>
+        <v>70.64</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10611,37 +10611,37 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>68.83</v>
+        <v>12.49</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>YLC</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>12.7</v>
+        <v>30.31</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -10651,17 +10651,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>30.19</v>
+        <v>12.11</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -10671,17 +10671,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>12.11</v>
+        <v>57.18</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -10691,30 +10691,10 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>57.3</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>YLC</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Yatırım Fonu Katılma Payı</t>
-        </is>
-      </c>
-      <c r="D59" t="n">
         <v>0.4</v>
       </c>
     </row>
@@ -10825,22 +10805,22 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>16.4</v>
+        <v>15.7</v>
       </c>
       <c r="E2" t="n">
-        <v>121.3</v>
+        <v>115.1</v>
       </c>
       <c r="F2" t="n">
-        <v>1223.5</v>
+        <v>1213.4</v>
       </c>
       <c r="G2" t="n">
-        <v>5843.8</v>
+        <v>5798.5</v>
       </c>
       <c r="H2" t="n">
-        <v>30.3</v>
+        <v>29.1</v>
       </c>
       <c r="I2" t="n">
-        <v>67.59999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="J2" t="n">
         <v>34.7</v>
@@ -10868,25 +10848,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>28.5</v>
+        <v>27.1</v>
       </c>
       <c r="E3" t="n">
-        <v>103.6</v>
+        <v>96.3</v>
       </c>
       <c r="F3" t="n">
-        <v>995.5</v>
+        <v>978.5</v>
       </c>
       <c r="G3" t="n">
-        <v>2605.6</v>
+        <v>2563.8</v>
       </c>
       <c r="H3" t="n">
-        <v>26.7</v>
+        <v>25.2</v>
       </c>
       <c r="I3" t="n">
-        <v>61.4</v>
+        <v>60.9</v>
       </c>
       <c r="J3" t="n">
-        <v>27.2</v>
+        <v>27.1</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -10911,25 +10891,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-12.1</v>
+        <v>-11.4</v>
       </c>
       <c r="E4" t="n">
-        <v>17.7</v>
+        <v>18.8</v>
       </c>
       <c r="F4" t="n">
-        <v>228</v>
+        <v>234.9</v>
       </c>
       <c r="G4" t="n">
-        <v>3238.2</v>
+        <v>3234.7</v>
       </c>
       <c r="H4" t="n">
-        <v>3.6</v>
+        <v>3.9</v>
       </c>
       <c r="I4" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="J4" t="n">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -10954,25 +10934,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>19</v>
+        <v>18.2</v>
       </c>
       <c r="E5" t="n">
-        <v>133.8</v>
+        <v>127.3</v>
       </c>
       <c r="F5" t="n">
-        <v>1351.6</v>
+        <v>1340.5</v>
       </c>
       <c r="G5" t="n">
-        <v>7450.9</v>
+        <v>7393.4</v>
       </c>
       <c r="H5" t="n">
-        <v>32.7</v>
+        <v>31.5</v>
       </c>
       <c r="I5" t="n">
-        <v>70.8</v>
+        <v>70.5</v>
       </c>
       <c r="J5" t="n">
-        <v>37.1</v>
+        <v>37</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -10997,25 +10977,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>28.5</v>
+        <v>27.1</v>
       </c>
       <c r="E6" t="n">
-        <v>103.6</v>
+        <v>96.3</v>
       </c>
       <c r="F6" t="n">
-        <v>995.5</v>
+        <v>978.5</v>
       </c>
       <c r="G6" t="n">
-        <v>2605.6</v>
+        <v>2563.8</v>
       </c>
       <c r="H6" t="n">
-        <v>26.7</v>
+        <v>25.2</v>
       </c>
       <c r="I6" t="n">
-        <v>61.4</v>
+        <v>60.9</v>
       </c>
       <c r="J6" t="n">
-        <v>27.2</v>
+        <v>27.1</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -11040,22 +11020,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-9.5</v>
+        <v>-8.9</v>
       </c>
       <c r="E7" t="n">
-        <v>30.2</v>
+        <v>31</v>
       </c>
       <c r="F7" t="n">
-        <v>356.1</v>
+        <v>362</v>
       </c>
       <c r="G7" t="n">
-        <v>4845.3</v>
+        <v>4829.6</v>
       </c>
       <c r="H7" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="I7" t="n">
-        <v>9.4</v>
+        <v>9.6</v>
       </c>
       <c r="J7" t="n">
         <v>9.9</v>
@@ -11132,10 +11112,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>30.3</v>
+        <v>29.1</v>
       </c>
       <c r="E2" t="n">
-        <v>26.7</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="3">
@@ -11155,10 +11135,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
-        <v>5.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="4">
@@ -11178,10 +11158,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>67.59999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>61.4</v>
+        <v>60.9</v>
       </c>
     </row>
     <row r="5">
@@ -11201,10 +11181,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>18.7</v>
+        <v>18.5</v>
       </c>
       <c r="E5" t="n">
-        <v>14.3</v>
+        <v>13.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Haftalik veri guncellemesi (test calistirmasi, 2026-07-31)
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -3392,7 +3392,7 @@
         <v>2026</v>
       </c>
       <c r="B39" s="8" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -9991,11 +9991,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Kamu Dış Borçlanma Araçları</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>3.12</v>
+        <v>96.88</v>
       </c>
     </row>
     <row r="24">
@@ -10011,11 +10011,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Özel Sektör Dış Borçlanma Araçları</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>96.88</v>
+        <v>3.12</v>
       </c>
     </row>
     <row r="25">
@@ -10535,7 +10535,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.6</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="51">
@@ -10555,7 +10555,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>14.88</v>
+        <v>15.12</v>
       </c>
     </row>
     <row r="52">
@@ -10575,7 +10575,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="53">
@@ -10595,7 +10595,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>70.64</v>
+        <v>70.16</v>
       </c>
     </row>
     <row r="54">
@@ -10615,7 +10615,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>12.49</v>
+        <v>12.69</v>
       </c>
     </row>
     <row r="55">

</xml_diff>

<commit_message>
Haftalik veri guncellemesi + Sayfa 24 F/K kaynagi MSCI Turkiye'ye gecti
- Turkiye F/K (eskiden "BIST-100 F/K", CEIC kaynakli) artik MSCI'nin kendi
  Turkiye endeksinden okunuyor - GOP/Dunya F/K ile ayni metodoloji, elma-elma
  kiyas (guncelle_degerleme_fk.py, page.tsx). Eski CEIC-vs-MSCI karsilastirmasi
  GOP'a gore sadece %2 iskonto gosteriyordu (iki farkli saglayicinin bilinen
  ~%7-8 sapma payindan kucuk, anlamsizdi); yeni rakamla %38 cikiyor.
- Peer_PE_Karsilastirma'daki Turkiye satiri duzeltildi: "0,2" gibi bozuk/donuk
  bir degerdi, artik diger 9 ulkeyle ayni otomatik MSCI akisinda (6,69).
- ANZ sayfasinin getiri tablosu/grafigi dogrulandi, degisiklik gerekmedi -
  dort bagimsiz kaynak (Excel, TEFAS fiyat serisi, Rasyonet raporu, canli
  TEFAS API sorgusu) fonun trailing 12 aylik %23 civarindaki getirisinde
  birlesiyor.
- Bugunun haftalik veri yenilemesi (fon fiyat serileri, TEFAS onbellegi) dahil.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1466,7 +1466,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>13775</v>
+        <v>13704</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>13000</v>
@@ -1490,7 +1490,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>47.37</v>
+        <v>47.76</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>54.7</v>
@@ -1514,7 +1514,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>54.28</v>
+        <v>55.19</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>63.4</v>
@@ -1538,7 +1538,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>7408</v>
+        <v>7758</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>7000</v>
@@ -1562,7 +1562,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>6282</v>
+        <v>6551</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>5800</v>
@@ -2991,22 +2991,22 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>BIST-100 F/K</t>
+          <t>Turkiye F/K</t>
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>18.3</v>
+        <v>10.95</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>18.61</v>
+        <v>17.72</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -3030,7 +3030,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>24.57</v>
+        <v>24.25</v>
       </c>
     </row>
     <row r="5">
@@ -3392,7 +3392,7 @@
         <v>2026</v>
       </c>
       <c r="B39" s="8" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -3450,7 +3450,7 @@
     <row r="8">
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -3459,13 +3459,13 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>20.01</v>
+        <v>20.32</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -3474,13 +3474,13 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>18.21</v>
+        <v>18.06</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -3489,13 +3489,13 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>13.82</v>
+        <v>14.03</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -3504,13 +3504,13 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>12.43</v>
+        <v>12.45</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -3519,13 +3519,13 @@
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>10.06</v>
+        <v>10.66</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -3534,13 +3534,13 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>8.98</v>
+        <v>9.74</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -3549,13 +3549,13 @@
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>8.390000000000001</v>
+        <v>9.390000000000001</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -3564,13 +3564,13 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>8.06</v>
+        <v>8.59</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -3579,18 +3579,22 @@
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>8</v>
+        <v>8.44</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="8" t="n"/>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Türkiye</t>
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>0.2</v>
+        <v>6.69</v>
       </c>
     </row>
     <row r="18">
@@ -4393,7 +4397,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B2" s="8" t="n">
@@ -5177,7 +5181,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>15.7</v>
+        <v>18.2</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5195,7 +5199,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>19.5</v>
+        <v>20.6</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5213,7 +5217,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>31.8</v>
+        <v>33.1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5231,7 +5235,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>38.9</v>
+        <v>43.8</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5249,7 +5253,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>27.1</v>
+        <v>30.7</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5267,7 +5271,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>28.6</v>
+        <v>29.6</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5285,7 +5289,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>29.7</v>
+        <v>37.6</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5321,7 +5325,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>45.9</v>
+        <v>44.1</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5339,7 +5343,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>47.1</v>
+        <v>47.2</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5357,7 +5361,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>38</v>
+        <v>35.7</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5375,7 +5379,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>52.5</v>
+        <v>64.5</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5393,7 +5397,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>22.7</v>
+        <v>38.7</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5411,7 +5415,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>45.6</v>
+        <v>50.9</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5429,7 +5433,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>38.9</v>
+        <v>47.7</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5447,7 +5451,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>32.7</v>
+        <v>40.4</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5465,7 +5469,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23.4</v>
+        <v>23.5</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5483,7 +5487,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5501,7 +5505,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>17.1</v>
+        <v>17.4</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -5519,7 +5523,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>32.1</v>
+        <v>31.8</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -5580,7 +5584,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>13.4</v>
+        <v>18.8</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5598,7 +5602,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12.1</v>
+        <v>16.5</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5616,7 +5620,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>29.7</v>
+        <v>37.1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5634,7 +5638,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>25.5</v>
+        <v>26.5</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5652,7 +5656,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>14.2</v>
+        <v>27.8</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5670,7 +5674,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>27.6</v>
+        <v>29.2</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5688,7 +5692,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>31.4</v>
+        <v>44.8</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5706,7 +5710,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>19.4</v>
+        <v>27.3</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5724,7 +5728,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>22.3</v>
+        <v>27.8</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5742,7 +5746,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>21.9</v>
+        <v>31.4</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5760,7 +5764,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>24</v>
+        <v>26.2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5778,7 +5782,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-1</v>
+        <v>6.7</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5796,7 +5800,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>11.4</v>
+        <v>13</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5814,7 +5818,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5832,7 +5836,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14.4</v>
+        <v>22.2</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5850,7 +5854,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.5</v>
+        <v>11.4</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5868,7 +5872,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>25.6</v>
+        <v>28</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5886,7 +5890,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>22.4</v>
+        <v>23.1</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5904,7 +5908,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>17.8</v>
+        <v>19.9</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -6855,7 +6859,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6869,16 +6873,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2.9</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6892,16 +6896,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8.699999999999999</v>
+        <v>7.6</v>
       </c>
       <c r="E3" t="n">
-        <v>10.2</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6915,16 +6919,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>19.2</v>
+        <v>18.1</v>
       </c>
       <c r="E4" t="n">
-        <v>19.5</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6938,7 +6942,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>45.9</v>
+        <v>44.1</v>
       </c>
       <c r="E5" t="n">
         <v>45.6</v>
@@ -6947,7 +6951,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6961,16 +6965,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>22.4</v>
+        <v>23.1</v>
       </c>
       <c r="E6" t="n">
-        <v>22.8</v>
+        <v>25.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6984,16 +6988,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-0.6</v>
+        <v>3.8</v>
       </c>
       <c r="E7" t="n">
-        <v>-7.4</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -7007,16 +7011,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>-2.1</v>
+        <v>2.7</v>
       </c>
       <c r="E8" t="n">
-        <v>-7</v>
+        <v>-3.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -7030,16 +7034,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -7053,16 +7057,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>29.7</v>
+        <v>37.6</v>
       </c>
       <c r="E10" t="n">
-        <v>27.1</v>
+        <v>30.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -7076,16 +7080,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>21.9</v>
+        <v>31.4</v>
       </c>
       <c r="E11" t="n">
-        <v>19.4</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -7099,16 +7103,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>5.2</v>
+        <v>2.3</v>
       </c>
       <c r="E12" t="n">
-        <v>6.8</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -7122,16 +7126,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>5.4</v>
+        <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>6.6</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7145,16 +7149,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>15.5</v>
+        <v>11.3</v>
       </c>
       <c r="E14" t="n">
-        <v>17.4</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -7168,16 +7172,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>38</v>
+        <v>35.7</v>
       </c>
       <c r="E15" t="n">
-        <v>42.6</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7191,16 +7195,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>27.6</v>
+        <v>29.2</v>
       </c>
       <c r="E16" t="n">
-        <v>32.3</v>
+        <v>28.3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -7214,16 +7218,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>-10.7</v>
+        <v>4.9</v>
       </c>
       <c r="E17" t="n">
-        <v>-1.3</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7237,16 +7241,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>9.699999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="E18" t="n">
-        <v>19.4</v>
+        <v>29.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7260,16 +7264,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>27.3</v>
+        <v>34.4</v>
       </c>
       <c r="E19" t="n">
-        <v>33.8</v>
+        <v>60.8</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7283,16 +7287,16 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>52.5</v>
+        <v>64.5</v>
       </c>
       <c r="E20" t="n">
-        <v>48.9</v>
+        <v>75.40000000000001</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7306,16 +7310,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>31.4</v>
+        <v>44.8</v>
       </c>
       <c r="E21" t="n">
-        <v>44.5</v>
+        <v>71.09999999999999</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7329,16 +7333,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>-2.2</v>
+        <v>12.5</v>
       </c>
       <c r="E22" t="n">
-        <v>-2.6</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7352,16 +7356,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>3.1</v>
+        <v>14.6</v>
       </c>
       <c r="E23" t="n">
-        <v>10.9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7375,16 +7379,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1.2</v>
+        <v>12.7</v>
       </c>
       <c r="E24" t="n">
-        <v>17.1</v>
+        <v>32.7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7398,16 +7402,16 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>22.7</v>
+        <v>38.7</v>
       </c>
       <c r="E25" t="n">
-        <v>37.2</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7421,16 +7425,16 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>14.2</v>
+        <v>27.8</v>
       </c>
       <c r="E26" t="n">
-        <v>31.6</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7444,16 +7448,16 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>5.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E27" t="n">
-        <v>-6.7</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7467,16 +7471,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>-2.3</v>
+        <v>-6.6</v>
       </c>
       <c r="E28" t="n">
-        <v>-17.4</v>
+        <v>-12.5</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7490,16 +7494,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>-0.4</v>
+        <v>3.2</v>
       </c>
       <c r="E29" t="n">
-        <v>-10.8</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7513,16 +7517,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>45.6</v>
+        <v>50.9</v>
       </c>
       <c r="E30" t="n">
-        <v>22.2</v>
+        <v>34.6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7536,16 +7540,16 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>25.5</v>
+        <v>26.5</v>
       </c>
       <c r="E31" t="n">
-        <v>7.1</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7559,16 +7563,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>-0.7</v>
+        <v>0.8</v>
       </c>
       <c r="E32" t="n">
-        <v>-1.6</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7582,16 +7586,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>-4.3</v>
+        <v>-2.7</v>
       </c>
       <c r="E33" t="n">
-        <v>-1.9</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7605,16 +7609,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>-1.7</v>
+        <v>-1.1</v>
       </c>
       <c r="E34" t="n">
-        <v>5.3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7628,16 +7632,16 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>19.5</v>
+        <v>20.6</v>
       </c>
       <c r="E35" t="n">
-        <v>28.6</v>
+        <v>29.6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7651,16 +7655,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>12.1</v>
+        <v>16.5</v>
       </c>
       <c r="E36" t="n">
-        <v>22.3</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7674,16 +7678,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4491.6</v>
+        <v>4669</v>
       </c>
       <c r="E37" t="n">
-        <v>4865.8</v>
+        <v>5090.4</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7697,16 +7701,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>-3.4</v>
+        <v>1.2</v>
       </c>
       <c r="E38" t="n">
-        <v>-7.4</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7720,16 +7724,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>-4.5</v>
+        <v>-3</v>
       </c>
       <c r="E39" t="n">
-        <v>-7</v>
+        <v>-3.9</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7743,16 +7747,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>-1.8</v>
+        <v>-0.2</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7766,16 +7770,16 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>15.7</v>
+        <v>18.2</v>
       </c>
       <c r="E41" t="n">
-        <v>27.1</v>
+        <v>30.7</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7789,16 +7793,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>13.4</v>
+        <v>18.8</v>
       </c>
       <c r="E42" t="n">
-        <v>19.4</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7812,16 +7816,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>5798.5</v>
+        <v>6078.8</v>
       </c>
       <c r="E43" t="n">
-        <v>2563.8</v>
+        <v>2740.7</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7835,16 +7839,16 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>115.1</v>
+        <v>100.5</v>
       </c>
       <c r="E44" t="n">
-        <v>96.3</v>
+        <v>96.40000000000001</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7858,16 +7862,16 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1213.4</v>
+        <v>1211.5</v>
       </c>
       <c r="E45" t="n">
-        <v>978.5</v>
+        <v>1006.7</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7881,16 +7885,16 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.5</v>
+        <v>2.3</v>
       </c>
       <c r="E46" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7904,16 +7908,16 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>5.1</v>
+        <v>1.7</v>
       </c>
       <c r="E47" t="n">
-        <v>3.6</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7927,16 +7931,16 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>11.3</v>
+        <v>17.6</v>
       </c>
       <c r="E48" t="n">
-        <v>18.9</v>
+        <v>24.2</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7950,16 +7954,16 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>38.9</v>
+        <v>43.8</v>
       </c>
       <c r="E49" t="n">
-        <v>48.7</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7973,16 +7977,16 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>29.7</v>
+        <v>37.1</v>
       </c>
       <c r="E50" t="n">
-        <v>38.9</v>
+        <v>47.6</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -7996,16 +8000,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>3.1</v>
+        <v>9</v>
       </c>
       <c r="E51" t="n">
-        <v>2.5</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -8019,16 +8023,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>-7.8</v>
+        <v>-3.3</v>
       </c>
       <c r="E52" t="n">
-        <v>-6.2</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -8042,16 +8046,16 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-13.9</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="E53" t="n">
-        <v>-10.3</v>
+        <v>-5.1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -8065,16 +8069,16 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>38.9</v>
+        <v>47.7</v>
       </c>
       <c r="E54" t="n">
-        <v>41.7</v>
+        <v>50</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -8088,16 +8092,16 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>-1</v>
+        <v>6.7</v>
       </c>
       <c r="E55" t="n">
-        <v>2.4</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -8111,13 +8115,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>-1.4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -8131,13 +8135,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>5.2</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -8151,13 +8155,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>12</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -8171,13 +8175,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>32.7</v>
+        <v>40.4</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -8191,13 +8195,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>14.4</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -8211,16 +8215,16 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="E61" t="n">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -8234,16 +8238,16 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>10.9</v>
+        <v>11.2</v>
       </c>
       <c r="E62" t="n">
-        <v>10.2</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -8257,16 +8261,16 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>22.4</v>
+        <v>22.8</v>
       </c>
       <c r="E63" t="n">
-        <v>20.9</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -8283,13 +8287,13 @@
         <v>50.2</v>
       </c>
       <c r="E64" t="n">
-        <v>47.1</v>
+        <v>47.2</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -8303,16 +8307,16 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>25.6</v>
+        <v>28</v>
       </c>
       <c r="E65" t="n">
-        <v>24</v>
+        <v>26.2</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -8326,7 +8330,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="E66" t="n">
         <v>0.2</v>
@@ -8335,7 +8339,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -8349,7 +8353,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>5.4</v>
+        <v>6.2</v>
       </c>
       <c r="E67" t="n">
         <v>0.6</v>
@@ -8358,7 +8362,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -8372,7 +8376,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>9.699999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="E68" t="n">
         <v>1.1</v>
@@ -8381,7 +8385,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -8395,16 +8399,16 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>23.4</v>
+        <v>23.5</v>
       </c>
       <c r="E69" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -8418,16 +8422,16 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>11.4</v>
+        <v>13</v>
       </c>
       <c r="E70" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -8441,13 +8445,13 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -8461,13 +8465,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>10.5</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -8481,7 +8485,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>21.3</v>
+        <v>21.7</v>
       </c>
     </row>
   </sheetData>
@@ -8544,7 +8548,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8569,7 +8573,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8588,13 +8592,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8613,13 +8617,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>9.300000000000001</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8638,13 +8642,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>17.1</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8663,13 +8667,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>10.5</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8688,13 +8692,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8713,13 +8717,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10.2</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8738,13 +8742,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>20.9</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8763,13 +8767,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>47.1</v>
+        <v>47.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -8788,13 +8792,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>24</v>
+        <v>26.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -8813,13 +8817,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>8.300000000000001</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -8838,13 +8842,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -8863,13 +8867,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>15.8</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -8888,13 +8892,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>37.1</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -8913,13 +8917,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>28.3</v>
+        <v>26.9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -8938,13 +8942,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>3.9</v>
+        <v>-7.9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -8963,13 +8967,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>12.4</v>
+        <v>-4.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -8988,13 +8992,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>20.4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9013,13 +9017,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>52.8</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9038,13 +9042,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>39.7</v>
+        <v>30.9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9063,13 +9067,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>-2.7</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9088,13 +9092,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>12.3</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9113,13 +9117,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>10</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9138,13 +9142,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>25</v>
+        <v>44.8</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9163,13 +9167,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>16</v>
+        <v>29.7</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -9188,13 +9192,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1.2</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -9213,13 +9217,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>32.6</v>
+        <v>49.3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -9238,13 +9242,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>78.09999999999999</v>
+        <v>123.1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -9263,13 +9267,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>93.3</v>
+        <v>132.2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -9288,13 +9292,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>97.40000000000001</v>
+        <v>147.8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -9313,13 +9317,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>3.44</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -9344,7 +9348,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -9363,13 +9367,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>22.21</v>
+        <v>22.41</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -9388,13 +9392,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>50.57</v>
+        <v>50.37</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -9413,7 +9417,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>26.01</v>
+        <v>28.16</v>
       </c>
     </row>
   </sheetData>
@@ -9527,7 +9531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9561,7 +9565,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9575,13 +9579,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>15.7</v>
+        <v>13.03</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9595,13 +9599,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>14.52</v>
+        <v>10.63</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9615,13 +9619,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.24</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9635,13 +9639,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2.57</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9655,13 +9659,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4.62</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9671,17 +9675,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Takasbank Para Piyasası</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>36.95</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9691,17 +9695,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>46.29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9711,57 +9715,57 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>19.4</v>
+        <v>4.31</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AAS</t>
+          <t>AAL</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5.63</v>
+        <v>19.75</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AAS</t>
+          <t>AAL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>77.39</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -9771,57 +9775,57 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>16.98</v>
+        <v>22.98</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AAV</t>
+          <t>AAS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>83.14</v>
+        <v>70.52</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AAV</t>
+          <t>AAS</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>13.32</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -9831,57 +9835,57 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3.54</v>
+        <v>86.31999999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>AED</t>
+          <t>AAV</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Devlet Tahvili</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.51</v>
+        <v>10.04</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AED</t>
+          <t>AAV</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3.54</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -9891,17 +9895,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Devlet Tahvili</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>65.08</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -9911,17 +9915,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1.12</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9931,17 +9935,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.68</v>
+        <v>58.13</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9951,17 +9955,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>15.31</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9971,37 +9975,37 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>12.76</v>
+        <v>22.42</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ANZ</t>
+          <t>AED</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Kamu Dış Borçlanma Araçları</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>96.88</v>
+        <v>14.28</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -10015,33 +10019,33 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3.12</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AYA</t>
+          <t>ANZ</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Özel Sektör Dış Borçlanma Araçları</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>81.31</v>
+        <v>98.34999999999999</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -10051,17 +10055,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.92</v>
+        <v>82.04000000000001</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -10071,17 +10075,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>3.79</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -10091,17 +10095,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2.88</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -10111,37 +10115,37 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>11.1</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DGH</t>
+          <t>AYA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1.58</v>
+        <v>11.04</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -10151,17 +10155,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.92</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -10171,17 +10175,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>38.28</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -10191,17 +10195,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1.23</v>
+        <v>20.92</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -10211,37 +10215,37 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>57.99</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>JET</t>
+          <t>DGH</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>22.01</v>
+        <v>76.15000000000001</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -10251,17 +10255,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1.82</v>
+        <v>22.19</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -10271,17 +10275,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>70.58</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -10291,57 +10295,57 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>5.59</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PKF</t>
+          <t>JET</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Kamu Kira Sertifikası (TL)</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>3.41</v>
+        <v>70.29000000000001</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PKF</t>
+          <t>JET</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Kıymetli Maden</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>94.84999999999999</v>
+        <v>5.93</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -10351,97 +10355,97 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Kamu Kira Sertifikası (TL)</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1.74</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PKP</t>
+          <t>PKF</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Katılma Hesabı (TL)</t>
+          <t>Kıymetli Maden</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>72.13</v>
+        <v>94.23999999999999</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PKP</t>
+          <t>PKF</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>27.87</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>RTG</t>
+          <t>PKP</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>20.76</v>
+        <v>76.54000000000001</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>RTG</t>
+          <t>PKP</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.82</v>
+        <v>23.46</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10451,17 +10455,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>66.09</v>
+        <v>21.42</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -10471,42 +10475,42 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>12.33</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TLZ</t>
+          <t>RTG</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>90.31</v>
+        <v>65.20999999999999</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TLZ</t>
+          <t>RTG</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -10515,53 +10519,53 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>9.69</v>
+        <v>12.22</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>TLZ</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.63</v>
+        <v>88.88</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>TLZ</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>15.12</v>
+        <v>11.12</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -10571,17 +10575,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.4</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -10591,17 +10595,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>70.16</v>
+        <v>14.08</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10611,77 +10615,77 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>12.69</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>YLC</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>30.31</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>YLC</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>12.11</v>
+        <v>70.19</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>YLC</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>57.18</v>
+        <v>11.37</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -10691,11 +10695,71 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
+          <t>Yerli Hisse Senedi</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>33.4</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>YLC</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>VİOP Teminatı</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>YLC</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Yabancı Hisse Senedi</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>62.46</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>YLC</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
           <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
-      <c r="D58" t="n">
-        <v>0.4</v>
+      <c r="D61" t="n">
+        <v>0.49</v>
       </c>
     </row>
   </sheetData>
@@ -10805,25 +10869,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>15.7</v>
+        <v>18.2</v>
       </c>
       <c r="E2" t="n">
-        <v>115.1</v>
+        <v>100.5</v>
       </c>
       <c r="F2" t="n">
-        <v>1213.4</v>
+        <v>1211.5</v>
       </c>
       <c r="G2" t="n">
-        <v>5798.5</v>
+        <v>6078.8</v>
       </c>
       <c r="H2" t="n">
-        <v>29.1</v>
+        <v>26.1</v>
       </c>
       <c r="I2" t="n">
-        <v>67.40000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="J2" t="n">
-        <v>34.7</v>
+        <v>35</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -10848,25 +10912,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>27.1</v>
+        <v>30.7</v>
       </c>
       <c r="E3" t="n">
-        <v>96.3</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>978.5</v>
+        <v>1006.7</v>
       </c>
       <c r="G3" t="n">
-        <v>2563.8</v>
+        <v>2740.7</v>
       </c>
       <c r="H3" t="n">
         <v>25.2</v>
       </c>
       <c r="I3" t="n">
-        <v>60.9</v>
+        <v>61.7</v>
       </c>
       <c r="J3" t="n">
-        <v>27.1</v>
+        <v>27.6</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -10891,25 +10955,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-11.4</v>
+        <v>-12.5</v>
       </c>
       <c r="E4" t="n">
-        <v>18.8</v>
+        <v>4.1</v>
       </c>
       <c r="F4" t="n">
-        <v>234.9</v>
+        <v>204.8</v>
       </c>
       <c r="G4" t="n">
-        <v>3234.7</v>
+        <v>3338.1</v>
       </c>
       <c r="H4" t="n">
-        <v>3.9</v>
+        <v>0.9</v>
       </c>
       <c r="I4" t="n">
-        <v>6.5</v>
+        <v>5.6</v>
       </c>
       <c r="J4" t="n">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -10934,25 +10998,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>18.2</v>
+        <v>20.8</v>
       </c>
       <c r="E5" t="n">
-        <v>127.3</v>
+        <v>111.9</v>
       </c>
       <c r="F5" t="n">
-        <v>1340.5</v>
+        <v>1338.4</v>
       </c>
       <c r="G5" t="n">
-        <v>7393.4</v>
+        <v>7749.4</v>
       </c>
       <c r="H5" t="n">
-        <v>31.5</v>
+        <v>28.4</v>
       </c>
       <c r="I5" t="n">
-        <v>70.5</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>37</v>
+        <v>37.3</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -10977,25 +11041,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>27.1</v>
+        <v>30.7</v>
       </c>
       <c r="E6" t="n">
-        <v>96.3</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>978.5</v>
+        <v>1006.7</v>
       </c>
       <c r="G6" t="n">
-        <v>2563.8</v>
+        <v>2740.7</v>
       </c>
       <c r="H6" t="n">
         <v>25.2</v>
       </c>
       <c r="I6" t="n">
-        <v>60.9</v>
+        <v>61.7</v>
       </c>
       <c r="J6" t="n">
-        <v>27.1</v>
+        <v>27.6</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -11020,25 +11084,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-8.9</v>
+        <v>-9.9</v>
       </c>
       <c r="E7" t="n">
-        <v>31</v>
+        <v>15.5</v>
       </c>
       <c r="F7" t="n">
-        <v>362</v>
+        <v>331.7</v>
       </c>
       <c r="G7" t="n">
-        <v>4829.6</v>
+        <v>5008.7</v>
       </c>
       <c r="H7" t="n">
-        <v>6.3</v>
+        <v>3.2</v>
       </c>
       <c r="I7" t="n">
-        <v>9.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>9.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -11112,7 +11176,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>29.1</v>
+        <v>26.1</v>
       </c>
       <c r="E2" t="n">
         <v>25.2</v>
@@ -11135,10 +11199,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>4.3</v>
       </c>
       <c r="E3" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="4">
@@ -11158,10 +11222,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>67.40000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="E4" t="n">
-        <v>60.9</v>
+        <v>61.7</v>
       </c>
     </row>
     <row r="5">
@@ -11181,10 +11245,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>18.5</v>
+        <v>18.6</v>
       </c>
       <c r="E5" t="n">
-        <v>13.9</v>
+        <v>14.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sayfa 2 ve iletisim sayfasi ekip guncellemesi: Etem Oztekin CEO oldu
- Fon Yonetimi org semasi (Sayfa 2): Batuhan Ozsahin (liderlik + Fon
  Yoneticileri) cikarildi, Etem Oztekin unvani "CEO, Board Member" oldu.
  Elmas Ozturk, Arastirma'dan Portfoy Yoneticisi Yardimcilari'na tasindi
  (Berk Tuna Subasi'nin altina).
- Iletisim sayfasi (son sayfa): ayni sekilde Batuhan Ozsahin cikarildi,
  Etem Oztekin unvani "CEO, Yonetim Kurulu Uyesi" oldu.
- Veri_Kaynagi.xlsx (Ekip_Organizasyon + Ekip sekmeleri) ve
  build_veri_kaynagi.py şema kaynagi birlikte guncellendi, /sunum
  render'i ekran goruntusuyle dogrulandi.
- Bekleyen haftalik veri yenilemesi (bist100_usd_endeksi.json) dahil.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1,38 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Kapak_Ozet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Fon_Katalog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Fon_Performans" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Fon_Performans_Ek_Kriter" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Fon_Fiyat_Serisi" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Fon_Portfoy_Dagilimi" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Fon_Getiri_Analizi_Detay" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Fon_Yillik_Getiri_Karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Fon_Temettu_Verimi" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Piyasa_Senaryolari" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Makro_Gostergeler" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Degerleme_CDS_MSCI" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Bist_Yillik_Getiriler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Peer_PE_Karsilastirma" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Fon_Metinleri" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Sabit_Metinler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Fon_Avantajlari_Maddeler" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Vergi_Bireysel_Fon_Listesi" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Vergi_ANZ_Tablosu" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Ekip" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Ekip_Organizasyon" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Ata_Fonlari_Performans_Ozet" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Ata_Fonlari_Performans_Ozet_YBB" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Yatirim_100TL_Dagilim" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Yatirim_100TL_Maddeler" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kapak_Ozet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Katalog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Performans" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Performans_Ek_Kriter" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Fiyat_Serisi" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Portfoy_Dagilimi" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Getiri_Analizi_Detay" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Yillik_Getiri_Karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Temettu_Verimi" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Piyasa_Senaryolari" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Makro_Gostergeler" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Degerleme_CDS_MSCI" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bist_Yillik_Getiriler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer_PE_Karsilastirma" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Metinleri" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sabit_Metinler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Avantajlari_Maddeler" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi_Bireysel_Fon_Listesi" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi_ANZ_Tablosu" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ekip" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ekip_Organizasyon" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ata_Fonlari_Performans_Ozet" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ata_Fonlari_Performans_Ozet_YBB" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatirim_100TL_Dagilim" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatirim_100TL_Maddeler" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>47.76</v>
+        <v>47.85</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>54.7</v>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>55.19</v>
+        <v>55.5</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>63.4</v>
@@ -3392,7 +3392,7 @@
         <v>2026</v>
       </c>
       <c r="B39" s="8" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -4582,112 +4582,96 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Batuhan Özşahin</t>
+          <t>Etem Öztekin</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>Co - CEO, CIO</t>
+          <t>CEO, Yönetim Kurulu Üyesi</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>0212 310 63 92</t>
+          <t>0212 310 63 85</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>batuhan.ozsahin@ataportfoy.com.tr</t>
+          <t>etem.oztekin@ataportfoy.com.tr</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>Etem Öztekin</t>
+          <t>Şebnem Kaya</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Co - CEO, Yönetim Kurulu Üyesi</t>
+          <t>Genel Müdür Yardımcısı</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>0212 310 63 85</t>
+          <t>0212 310 63 75</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>etem.oztekin@ataportfoy.com.tr</t>
+          <t>skaya@ataportfoy.com.tr</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Şebnem Kaya</t>
+          <t>Funda Sevgi Tunal</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Genel Müdür Yardımcısı</t>
+          <t>Direktör</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>0212 310 63 75</t>
+          <t>0212 310 60 21</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>skaya@ataportfoy.com.tr</t>
+          <t>funda.tunal@ataportfoy.com.tr</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Funda Sevgi Tunal</t>
+          <t>Bade Miray Süngü</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Direktör</t>
+          <t>Müdür Yardımcısı</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>0212 310 60 21</t>
+          <t>0212 310 60 38</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>funda.tunal@ataportfoy.com.tr</t>
+          <t>bade.sungu@ataportfoy.com.tr</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>Bade Miray Süngü</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Müdür Yardımcısı</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>0212 310 60 38</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>bade.sungu@ataportfoy.com.tr</t>
-        </is>
-      </c>
+      <c r="A6" s="8" t="n"/>
+      <c r="B6" s="8" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4738,15 +4722,15 @@
           <t>Fon Yönetimi</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr"/>
+      <c r="B2" s="8" t="n"/>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Batuhan Özşahin</t>
+          <t>Etem Öztekin</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>Co-CEO, CIO</t>
+          <t>CEO, Board Member</t>
         </is>
       </c>
     </row>
@@ -4756,17 +4740,17 @@
           <t>Fon Yönetimi</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr"/>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Fon Yöneticileri</t>
+        </is>
+      </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Etem Öztekin</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Co-CEO, Board Member</t>
-        </is>
-      </c>
+          <t>Suna Tanrıverdi Fidan</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -4781,10 +4765,10 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Batuhan Özşahin</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr"/>
+          <t>Farshad Mirzazadeh, CFA</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -4799,10 +4783,10 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Suna Tanrıverdi Fidan</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr"/>
+          <t>Samet Zağlı</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -4812,15 +4796,15 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Fon Yöneticileri</t>
+          <t>Portföy Yöneticisi Yardımcıları</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Farshad Mirzazadeh, CFA</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr"/>
+          <t>Berk Tuna Subaşı</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -4830,15 +4814,15 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Fon Yöneticileri</t>
+          <t>Portföy Yöneticisi Yardımcıları</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Samet Zağlı</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr"/>
+          <t>Elmas Öztürk</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -4848,15 +4832,15 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Portföy Yöneticisi Yardımcıları</t>
+          <t>Araştırma</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Berk Tuna Subaşı</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr"/>
+          <t>Batuhan Demirci</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -4866,15 +4850,15 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Araştırma</t>
+          <t>Varlık Yönetimi ve Yatırım Danışmanlığı</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Elmas Öztürk</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr"/>
+          <t>Şebnem Kaya</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -4884,15 +4868,15 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Araştırma</t>
+          <t>Varlık Yönetimi ve Yatırım Danışmanlığı</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Batuhan Demirci</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr"/>
+          <t>Funda Sevgi Tunal</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -4907,10 +4891,10 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Şebnem Kaya</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr"/>
+          <t>Bade Miray Süngü</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -4925,46 +4909,46 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Funda Sevgi Tunal</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr"/>
+          <t>Mete Tezel</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Fon Yönetimi</t>
+          <t>Fon Operasyon</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Varlık Yönetimi ve Yatırım Danışmanlığı</t>
+          <t>Fon Operasyon</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Bade Miray Süngü</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr"/>
+          <t>Niyazi Takmaz</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Fon Yönetimi</t>
+          <t>Fon Operasyon</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Varlık Yönetimi ve Yatırım Danışmanlığı</t>
+          <t>Fon Operasyon</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Mete Tezel</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr"/>
+          <t>Güney Özütutar</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -4979,10 +4963,10 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Niyazi Takmaz</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr"/>
+          <t>Aslı Serin</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -4992,15 +4976,15 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Fon Operasyon</t>
+          <t>Risk Yönetimi</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Güney Özütutar</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr"/>
+          <t>Seyhan Dönmezkuş</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -5010,15 +4994,15 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Fon Operasyon</t>
+          <t>İç Kontrol</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Aslı Serin</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr"/>
+          <t>Sema Zorbacı</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -5028,15 +5012,15 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Risk Yönetimi</t>
+          <t>Teftiş</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Seyhan Dönmezkuş</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr"/>
+          <t>Gökhan Küçüoğlu</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -5046,15 +5030,15 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>İç Kontrol</t>
+          <t>İnsan Kaynakları</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Sema Zorbacı</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr"/>
+          <t>Yaren Telatar</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -5064,15 +5048,15 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Teftiş</t>
+          <t>Bilgi İşlem</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Gökhan Küçüoğlu</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr"/>
+          <t>Kadir Mert Adnan</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -5082,51 +5066,27 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>İnsan Kaynakları</t>
+          <t>Muhasebe</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Yaren Telatar</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr"/>
+          <t>Meltem Ayrım</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Fon Operasyon</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Bilgi İşlem</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Kadir Mert Adnan</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr"/>
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>Fon Operasyon</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Muhasebe</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Meltem Ayrım</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr"/>
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Bade Miray Sungu sunumdan cikarildi + haftalik veri guncellemesi
- Sayfa 2 (Fon Yonetimi org semasi, Varlik Yonetimi ve Yatirim
  Danismanligi bolumu) ve iletisim sayfasindan Bade Miray Sungu
  cikarildi. Veri_Kaynagi.xlsx + build_veri_kaynagi.py birlikte
  guncellendi, /sunum render'i ekran goruntusuyle dogrulandi.
- Bu oturum sirasinda tetiklenen haftalik veri yenilemesi (fon fiyat
  serileri, Turkiye CDS, TEFAS ANZ onbellegi) dahil edildi.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1466,7 +1466,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>13704</v>
+        <v>14128</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>13000</v>
@@ -1490,7 +1490,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>47.85</v>
+        <v>47.92</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>54.7</v>
@@ -1514,7 +1514,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>55.5</v>
+        <v>56.07</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>63.4</v>
@@ -1538,7 +1538,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>7758</v>
+        <v>7786</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>7000</v>
@@ -1562,7 +1562,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>6551</v>
+        <v>6468</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>5800</v>
@@ -3392,7 +3392,7 @@
         <v>2026</v>
       </c>
       <c r="B39" s="8" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -4397,7 +4397,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B2" s="8" t="n">
@@ -4646,26 +4646,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Bade Miray Süngü</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>Müdür Yardımcısı</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>0212 310 60 38</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>bade.sungu@ataportfoy.com.tr</t>
-        </is>
-      </c>
+      <c r="A5" s="8" t="n"/>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n"/>
@@ -4891,7 +4875,7 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Bade Miray Süngü</t>
+          <t>Mete Tezel</t>
         </is>
       </c>
       <c r="D11" s="8" t="n"/>
@@ -4899,17 +4883,17 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Fon Yönetimi</t>
+          <t>Fon Operasyon</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Varlık Yönetimi ve Yatırım Danışmanlığı</t>
+          <t>Fon Operasyon</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Mete Tezel</t>
+          <t>Niyazi Takmaz</t>
         </is>
       </c>
       <c r="D12" s="8" t="n"/>
@@ -4927,7 +4911,7 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Niyazi Takmaz</t>
+          <t>Güney Özütutar</t>
         </is>
       </c>
       <c r="D13" s="8" t="n"/>
@@ -4945,7 +4929,7 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Güney Özütutar</t>
+          <t>Aslı Serin</t>
         </is>
       </c>
       <c r="D14" s="8" t="n"/>
@@ -4958,12 +4942,12 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Fon Operasyon</t>
+          <t>Risk Yönetimi</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Aslı Serin</t>
+          <t>Seyhan Dönmezkuş</t>
         </is>
       </c>
       <c r="D15" s="8" t="n"/>
@@ -4976,12 +4960,12 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Risk Yönetimi</t>
+          <t>İç Kontrol</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Seyhan Dönmezkuş</t>
+          <t>Sema Zorbacı</t>
         </is>
       </c>
       <c r="D16" s="8" t="n"/>
@@ -4994,12 +4978,12 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>İç Kontrol</t>
+          <t>Teftiş</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Sema Zorbacı</t>
+          <t>Gökhan Küçüoğlu</t>
         </is>
       </c>
       <c r="D17" s="8" t="n"/>
@@ -5012,12 +4996,12 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Teftiş</t>
+          <t>İnsan Kaynakları</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Gökhan Küçüoğlu</t>
+          <t>Yaren Telatar</t>
         </is>
       </c>
       <c r="D18" s="8" t="n"/>
@@ -5030,12 +5014,12 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>İnsan Kaynakları</t>
+          <t>Bilgi İşlem</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Yaren Telatar</t>
+          <t>Kadir Mert Adnan</t>
         </is>
       </c>
       <c r="D19" s="8" t="n"/>
@@ -5048,32 +5032,20 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Bilgi İşlem</t>
+          <t>Muhasebe</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Kadir Mert Adnan</t>
+          <t>Meltem Ayrım</t>
         </is>
       </c>
       <c r="D20" s="8" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>Fon Operasyon</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Muhasebe</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Meltem Ayrım</t>
-        </is>
-      </c>
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
       <c r="D21" s="8" t="n"/>
     </row>
     <row r="22">
@@ -5141,7 +5113,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>18.2</v>
+        <v>25</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5159,7 +5131,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.6</v>
+        <v>24.4</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5177,7 +5149,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>33.1</v>
+        <v>37.2</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5195,7 +5167,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>43.8</v>
+        <v>53</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5213,7 +5185,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>30.7</v>
+        <v>35.1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5231,7 +5203,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>29.6</v>
+        <v>38.6</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5249,7 +5221,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>37.6</v>
+        <v>43</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5267,7 +5239,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>50.2</v>
+        <v>50.1</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5303,7 +5275,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>47.2</v>
+        <v>47.1</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5321,7 +5293,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>35.7</v>
+        <v>37.5</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5339,7 +5311,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>64.5</v>
+        <v>61</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5357,7 +5329,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>38.7</v>
+        <v>32.6</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5375,7 +5347,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>50.9</v>
+        <v>52.5</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5393,7 +5365,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>47.7</v>
+        <v>54.8</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5411,7 +5383,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>40.4</v>
+        <v>37.4</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5429,7 +5401,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23.5</v>
+        <v>22.6</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5447,7 +5419,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5.1</v>
+        <v>4.5</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5465,7 +5437,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>17.4</v>
+        <v>17.3</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -5544,7 +5516,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>18.8</v>
+        <v>22.4</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5562,7 +5534,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>16.5</v>
+        <v>19.1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5580,7 +5552,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>37.1</v>
+        <v>42.2</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5598,7 +5570,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>26.5</v>
+        <v>27.4</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5616,7 +5588,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>27.8</v>
+        <v>23.8</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5634,7 +5606,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>29.2</v>
+        <v>31.2</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5652,7 +5624,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>44.8</v>
+        <v>41.9</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5670,7 +5642,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>27.3</v>
+        <v>30.4</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5688,7 +5660,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>27.8</v>
+        <v>34</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5706,7 +5678,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>31.4</v>
+        <v>34.7</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5724,7 +5696,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>26.2</v>
+        <v>27.2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5742,7 +5714,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>6.7</v>
+        <v>12.1</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5760,7 +5732,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13</v>
+        <v>13.3</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5778,7 +5750,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5796,7 +5768,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>22.2</v>
+        <v>21.3</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5814,7 +5786,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>11.4</v>
+        <v>11.7</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5832,7 +5804,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5850,7 +5822,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>23.1</v>
+        <v>24</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -6819,7 +6791,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6836,13 +6808,13 @@
         <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6856,16 +6828,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="E3" t="n">
-        <v>10.6</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6888,7 +6860,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6911,7 +6883,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6925,16 +6897,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>23.1</v>
+        <v>24</v>
       </c>
       <c r="E6" t="n">
-        <v>25.1</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6948,16 +6920,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3.8</v>
+        <v>5.8</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.5</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6971,16 +6943,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2.7</v>
+        <v>8.9</v>
       </c>
       <c r="E8" t="n">
-        <v>-3.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6994,16 +6966,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="E9" t="n">
-        <v>3.9</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -7017,16 +6989,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>37.6</v>
+        <v>43</v>
       </c>
       <c r="E10" t="n">
-        <v>30.7</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -7040,16 +7012,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>31.4</v>
+        <v>34.7</v>
       </c>
       <c r="E11" t="n">
-        <v>27.3</v>
+        <v>30.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -7063,16 +7035,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2.3</v>
+        <v>1.2</v>
       </c>
       <c r="E12" t="n">
-        <v>-2</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -7086,16 +7058,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>7.2</v>
       </c>
       <c r="E13" t="n">
-        <v>-1.1</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7109,16 +7081,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="E14" t="n">
-        <v>6.3</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -7132,16 +7104,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>35.7</v>
+        <v>37.5</v>
       </c>
       <c r="E15" t="n">
-        <v>35.7</v>
+        <v>40.6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7155,16 +7127,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>29.2</v>
+        <v>31.2</v>
       </c>
       <c r="E16" t="n">
-        <v>28.3</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -7178,16 +7150,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4.9</v>
+        <v>1.3</v>
       </c>
       <c r="E17" t="n">
-        <v>16.6</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7201,16 +7173,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>8.1</v>
+        <v>7.2</v>
       </c>
       <c r="E18" t="n">
-        <v>29.1</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7224,16 +7196,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>34.4</v>
+        <v>40.7</v>
       </c>
       <c r="E19" t="n">
-        <v>60.8</v>
+        <v>43.1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7247,16 +7219,16 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>64.5</v>
+        <v>61</v>
       </c>
       <c r="E20" t="n">
-        <v>75.40000000000001</v>
+        <v>54.8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7270,16 +7242,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>44.8</v>
+        <v>41.9</v>
       </c>
       <c r="E21" t="n">
-        <v>71.09999999999999</v>
+        <v>53.2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7293,16 +7265,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>12.5</v>
+        <v>5.3</v>
       </c>
       <c r="E22" t="n">
-        <v>12.4</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7316,16 +7288,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>14.6</v>
+        <v>12.4</v>
       </c>
       <c r="E23" t="n">
-        <v>16</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7339,16 +7311,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>12.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E24" t="n">
-        <v>32.7</v>
+        <v>20.7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7362,16 +7334,16 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>38.7</v>
+        <v>32.6</v>
       </c>
       <c r="E25" t="n">
-        <v>54</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7385,16 +7357,16 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>27.8</v>
+        <v>23.8</v>
       </c>
       <c r="E26" t="n">
-        <v>48</v>
+        <v>39.6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7408,16 +7380,16 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>9.699999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="E27" t="n">
-        <v>8.9</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7431,16 +7403,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>-6.6</v>
+        <v>1.8</v>
       </c>
       <c r="E28" t="n">
-        <v>-12.5</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7454,16 +7426,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>3.2</v>
+        <v>8.5</v>
       </c>
       <c r="E29" t="n">
-        <v>-2.5</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7477,16 +7449,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>50.9</v>
+        <v>52.5</v>
       </c>
       <c r="E30" t="n">
-        <v>34.6</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7500,16 +7472,16 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>26.5</v>
+        <v>27.4</v>
       </c>
       <c r="E31" t="n">
-        <v>17.5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7523,16 +7495,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.8</v>
+        <v>2.5</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7546,16 +7518,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>-2.7</v>
+        <v>2.9</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.4</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7569,16 +7541,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>-1.1</v>
+        <v>-2.1</v>
       </c>
       <c r="E34" t="n">
-        <v>5</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7592,16 +7564,16 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>20.6</v>
+        <v>24.4</v>
       </c>
       <c r="E35" t="n">
-        <v>29.6</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7615,16 +7587,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>16.5</v>
+        <v>19.1</v>
       </c>
       <c r="E36" t="n">
-        <v>27.8</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7638,16 +7610,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4669</v>
+        <v>4775.2</v>
       </c>
       <c r="E37" t="n">
-        <v>5090.4</v>
+        <v>5340.2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7661,16 +7633,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1.2</v>
+        <v>4.8</v>
       </c>
       <c r="E38" t="n">
-        <v>-0.5</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7684,16 +7656,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>-3</v>
+        <v>3.2</v>
       </c>
       <c r="E39" t="n">
-        <v>-3.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7707,16 +7679,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="E40" t="n">
-        <v>3.9</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7730,16 +7702,16 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>18.2</v>
+        <v>25</v>
       </c>
       <c r="E41" t="n">
-        <v>30.7</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7753,16 +7725,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>18.8</v>
+        <v>22.4</v>
       </c>
       <c r="E42" t="n">
-        <v>27.3</v>
+        <v>30.4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7776,16 +7748,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>6078.8</v>
+        <v>6264.8</v>
       </c>
       <c r="E43" t="n">
-        <v>2740.7</v>
+        <v>2809.4</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7799,16 +7771,16 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>100.5</v>
+        <v>109.5</v>
       </c>
       <c r="E44" t="n">
-        <v>96.40000000000001</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7822,16 +7794,16 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1211.5</v>
+        <v>1239.1</v>
       </c>
       <c r="E45" t="n">
-        <v>1006.7</v>
+        <v>1035.8</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7845,16 +7817,16 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2.3</v>
+        <v>4.9</v>
       </c>
       <c r="E46" t="n">
-        <v>2.8</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7868,16 +7840,16 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.7</v>
+        <v>6.7</v>
       </c>
       <c r="E47" t="n">
-        <v>2.5</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7891,16 +7863,16 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>17.6</v>
+        <v>18.7</v>
       </c>
       <c r="E48" t="n">
-        <v>24.2</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7914,16 +7886,16 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>43.8</v>
+        <v>53</v>
       </c>
       <c r="E49" t="n">
-        <v>54.5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7937,16 +7909,16 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>37.1</v>
+        <v>42.2</v>
       </c>
       <c r="E50" t="n">
-        <v>47.6</v>
+        <v>55.7</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -7960,16 +7932,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>9</v>
+        <v>12.6</v>
       </c>
       <c r="E51" t="n">
-        <v>8.699999999999999</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -7983,16 +7955,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>-3.3</v>
+        <v>6.2</v>
       </c>
       <c r="E52" t="n">
-        <v>-1.8</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -8006,16 +7978,16 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-8.300000000000001</v>
+        <v>-2.7</v>
       </c>
       <c r="E53" t="n">
-        <v>-5.1</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -8029,16 +8001,16 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>47.7</v>
+        <v>54.8</v>
       </c>
       <c r="E54" t="n">
-        <v>50</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -8052,16 +8024,16 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>6.7</v>
+        <v>12.1</v>
       </c>
       <c r="E55" t="n">
-        <v>10.4</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -8075,13 +8047,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>5</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -8095,13 +8067,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>7.6</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -8115,13 +8087,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>18.7</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -8135,13 +8107,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>40.4</v>
+        <v>37.4</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -8155,13 +8127,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>22.2</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -8184,7 +8156,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -8198,16 +8170,16 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>11.2</v>
+        <v>11.1</v>
       </c>
       <c r="E62" t="n">
-        <v>10.6</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -8224,13 +8196,13 @@
         <v>22.8</v>
       </c>
       <c r="E63" t="n">
-        <v>21.2</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -8244,16 +8216,16 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>50.2</v>
+        <v>50.1</v>
       </c>
       <c r="E64" t="n">
-        <v>47.2</v>
+        <v>47.1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -8267,16 +8239,16 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E65" t="n">
-        <v>26.2</v>
+        <v>27.2</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -8290,7 +8262,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="E66" t="n">
         <v>0.2</v>
@@ -8299,7 +8271,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -8313,7 +8285,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="E67" t="n">
         <v>0.6</v>
@@ -8322,7 +8294,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -8336,16 +8308,16 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>10.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E68" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -8359,7 +8331,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>23.5</v>
+        <v>22.6</v>
       </c>
       <c r="E69" t="n">
         <v>2.1</v>
@@ -8368,7 +8340,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -8382,16 +8354,16 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>13</v>
+        <v>13.3</v>
       </c>
       <c r="E70" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -8411,7 +8383,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -8425,13 +8397,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -8445,7 +8417,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
     </row>
   </sheetData>
@@ -8508,7 +8480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8533,7 +8505,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8552,13 +8524,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8577,13 +8549,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>9.6</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8602,13 +8574,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>17.4</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8627,13 +8599,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>11.4</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8658,7 +8630,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8677,13 +8649,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10.6</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8702,13 +8674,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>21.2</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8727,13 +8699,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>47.2</v>
+        <v>47.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -8752,13 +8724,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>26.2</v>
+        <v>27.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -8777,13 +8749,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1.2</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -8802,13 +8774,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.7</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -8827,13 +8799,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>5.4</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -8852,13 +8824,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>36.5</v>
+        <v>39.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -8877,13 +8849,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>26.9</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -8902,13 +8874,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>-7.9</v>
+        <v>-7.1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -8927,13 +8899,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>-4.4</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -8952,13 +8924,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>8</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -8977,13 +8949,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>34.3</v>
+        <v>41.9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9002,13 +8974,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>30.9</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9027,13 +8999,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>11.8</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9052,13 +9024,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>18.3</v>
+        <v>16.4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9077,13 +9049,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>27.3</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9102,13 +9074,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>44.8</v>
+        <v>38.4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9127,13 +9099,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>29.7</v>
+        <v>28.8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -9152,13 +9124,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>25.5</v>
+        <v>-4.4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -9177,13 +9149,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>49.3</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -9202,13 +9174,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>123.1</v>
+        <v>66.3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -9227,13 +9199,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>132.2</v>
+        <v>85.09999999999999</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -9252,13 +9224,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>147.8</v>
+        <v>98.40000000000001</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -9277,13 +9249,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>3.56</v>
+        <v>3.44</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -9302,13 +9274,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>10.79</v>
+        <v>10.77</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -9327,13 +9299,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>22.41</v>
+        <v>22.49</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -9352,13 +9324,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>50.37</v>
+        <v>50.25</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -9377,7 +9349,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>28.16</v>
+        <v>29.17</v>
       </c>
     </row>
   </sheetData>
@@ -9491,7 +9463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9525,7 +9497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9539,13 +9511,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>13.03</v>
+        <v>9.24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9559,13 +9531,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>10.63</v>
+        <v>10.89</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9575,17 +9547,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Kamu Kira Sertifikası (TL)</t>
+          <t>Hazine Bonosu</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.3</v>
+        <v>3.09</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9595,17 +9567,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Kamu Kira Sertifikası (TL)</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.26</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9615,17 +9587,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.42</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9635,17 +9607,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Takasbank Para Piyasası</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.95</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9655,17 +9627,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Takasbank Para Piyasası</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>46.29</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9675,17 +9647,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>4.31</v>
+        <v>48.48</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -9695,17 +9667,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>19.75</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -9715,22 +9687,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.06</v>
+        <v>19.86</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AAS</t>
+          <t>AAL</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -9739,13 +9711,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>22.98</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -9755,17 +9727,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>70.52</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -9775,37 +9747,37 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>6.5</v>
+        <v>39.86</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>AAV</t>
+          <t>AAS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>86.31999999999999</v>
+        <v>59.48</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -9815,17 +9787,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>10.04</v>
+        <v>92.27</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9835,37 +9807,37 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3.64</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AED</t>
+          <t>AAV</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Devlet Tahvili</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.51</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -9875,17 +9847,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Devlet Tahvili</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3.54</v>
+        <v>5.42</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9895,17 +9867,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>58.13</v>
+        <v>3.33</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9915,17 +9887,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1.12</v>
+        <v>55.41</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9935,17 +9907,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>22.42</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9955,22 +9927,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>14.28</v>
+        <v>3.09</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ANZ</t>
+          <t>AED</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -9979,73 +9951,73 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1.65</v>
+        <v>18.83</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ANZ</t>
+          <t>AED</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Özel Sektör Dış Borçlanma Araçları</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>98.34999999999999</v>
+        <v>12.87</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AYA</t>
+          <t>ANZ</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>82.04000000000001</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AYA</t>
+          <t>ANZ</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Özel Sektör Dış Borçlanma Araçları</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.92</v>
+        <v>98.12</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -10055,17 +10027,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3.64</v>
+        <v>85.7</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -10075,17 +10047,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2.36</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -10095,57 +10067,57 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>11.04</v>
+        <v>2.21</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DGH</t>
+          <t>AYA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1.03</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DGH</t>
+          <t>AYA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.8100000000000001</v>
+        <v>11.01</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -10155,17 +10127,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>20.92</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -10175,17 +10147,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1.09</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -10195,42 +10167,42 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>76.15000000000001</v>
+        <v>22.39</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>JET</t>
+          <t>DGH</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>22.19</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>JET</t>
+          <t>DGH</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -10239,13 +10211,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1.45</v>
+        <v>74.76000000000001</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -10255,17 +10227,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.14</v>
+        <v>23.42</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -10275,17 +10247,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>70.29000000000001</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -10295,57 +10267,57 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>5.93</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PKF</t>
+          <t>JET</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Kamu Kira Sertifikası (TL)</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>3.37</v>
+        <v>67.17</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PKF</t>
+          <t>JET</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Kıymetli Maden</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>94.23999999999999</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -10355,97 +10327,97 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Kamu Kira Sertifikası (TL)</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2.39</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PKP</t>
+          <t>PKF</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Katılma Hesabı (TL)</t>
+          <t>Kıymetli Maden</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>76.54000000000001</v>
+        <v>94.68000000000001</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PKP</t>
+          <t>PKF</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>23.46</v>
+        <v>2.08</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>RTG</t>
+          <t>PKP</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>21.42</v>
+        <v>78.22</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>RTG</t>
+          <t>PKP</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.15</v>
+        <v>21.78</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -10455,17 +10427,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>65.20999999999999</v>
+        <v>22.62</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -10475,42 +10447,42 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>12.22</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TLZ</t>
+          <t>RTG</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>88.88</v>
+        <v>64.47</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TLZ</t>
+          <t>RTG</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -10519,53 +10491,53 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>11.12</v>
+        <v>12.39</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>TLZ</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>1.39</v>
+        <v>88.77</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>TLZ</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>14.08</v>
+        <v>11.23</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10575,17 +10547,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>2.78</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -10595,17 +10567,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.19</v>
+        <v>14.71</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -10615,17 +10587,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>70.19</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -10635,57 +10607,57 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>11.37</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>YLC</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>33.4</v>
+        <v>71.8</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>YLC</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>3.65</v>
+        <v>10.81</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -10695,17 +10667,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>62.46</v>
+        <v>31.25</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -10715,11 +10687,51 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
+          <t>VİOP Teminatı</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>YLC</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Yabancı Hisse Senedi</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>67.45999999999999</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>YLC</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
           <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
-      <c r="D61" t="n">
-        <v>0.49</v>
+      <c r="D63" t="n">
+        <v>0.48</v>
       </c>
     </row>
   </sheetData>
@@ -10829,25 +10841,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>18.2</v>
+        <v>25</v>
       </c>
       <c r="E2" t="n">
-        <v>100.5</v>
+        <v>109.5</v>
       </c>
       <c r="F2" t="n">
-        <v>1211.5</v>
+        <v>1239.1</v>
       </c>
       <c r="G2" t="n">
-        <v>6078.8</v>
+        <v>6264.8</v>
       </c>
       <c r="H2" t="n">
-        <v>26.1</v>
+        <v>28</v>
       </c>
       <c r="I2" t="n">
-        <v>67.3</v>
+        <v>68</v>
       </c>
       <c r="J2" t="n">
-        <v>35</v>
+        <v>35.2</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -10872,25 +10884,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>30.7</v>
+        <v>35.1</v>
       </c>
       <c r="E3" t="n">
-        <v>96.40000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>1006.7</v>
+        <v>1035.8</v>
       </c>
       <c r="G3" t="n">
-        <v>2740.7</v>
+        <v>2809.4</v>
       </c>
       <c r="H3" t="n">
-        <v>25.2</v>
+        <v>25.8</v>
       </c>
       <c r="I3" t="n">
-        <v>61.7</v>
+        <v>62.6</v>
       </c>
       <c r="J3" t="n">
-        <v>27.6</v>
+        <v>27.7</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -10915,25 +10927,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-12.5</v>
+        <v>-10.1</v>
       </c>
       <c r="E4" t="n">
-        <v>4.1</v>
+        <v>10.4</v>
       </c>
       <c r="F4" t="n">
-        <v>204.8</v>
+        <v>203.3</v>
       </c>
       <c r="G4" t="n">
-        <v>3338.1</v>
+        <v>3455.4</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9</v>
+        <v>2.2</v>
       </c>
       <c r="I4" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="J4" t="n">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -10958,25 +10970,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>20.8</v>
+        <v>27.7</v>
       </c>
       <c r="E5" t="n">
-        <v>111.9</v>
+        <v>121.4</v>
       </c>
       <c r="F5" t="n">
-        <v>1338.4</v>
+        <v>1368.7</v>
       </c>
       <c r="G5" t="n">
-        <v>7749.4</v>
+        <v>7985.7</v>
       </c>
       <c r="H5" t="n">
-        <v>28.4</v>
+        <v>30.3</v>
       </c>
       <c r="I5" t="n">
-        <v>70.40000000000001</v>
+        <v>71.2</v>
       </c>
       <c r="J5" t="n">
-        <v>37.3</v>
+        <v>37.6</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -11001,25 +11013,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>30.7</v>
+        <v>35.1</v>
       </c>
       <c r="E6" t="n">
-        <v>96.40000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>1006.7</v>
+        <v>1035.8</v>
       </c>
       <c r="G6" t="n">
-        <v>2740.7</v>
+        <v>2809.4</v>
       </c>
       <c r="H6" t="n">
-        <v>25.2</v>
+        <v>25.8</v>
       </c>
       <c r="I6" t="n">
-        <v>61.7</v>
+        <v>62.6</v>
       </c>
       <c r="J6" t="n">
-        <v>27.6</v>
+        <v>27.7</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -11044,25 +11056,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-9.9</v>
+        <v>-7.4</v>
       </c>
       <c r="E7" t="n">
-        <v>15.5</v>
+        <v>22.3</v>
       </c>
       <c r="F7" t="n">
-        <v>331.7</v>
+        <v>332.9</v>
       </c>
       <c r="G7" t="n">
-        <v>5008.7</v>
+        <v>5176.3</v>
       </c>
       <c r="H7" t="n">
-        <v>3.2</v>
+        <v>4.5</v>
       </c>
       <c r="I7" t="n">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="J7" t="n">
-        <v>9.699999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -11136,10 +11148,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>26.1</v>
+        <v>28</v>
       </c>
       <c r="E2" t="n">
-        <v>25.2</v>
+        <v>25.8</v>
       </c>
     </row>
     <row r="3">
@@ -11159,10 +11171,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4.3</v>
+        <v>5.9</v>
       </c>
       <c r="E3" t="n">
-        <v>3.6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="4">
@@ -11182,10 +11194,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>67.3</v>
+        <v>68</v>
       </c>
       <c r="E4" t="n">
-        <v>61.7</v>
+        <v>62.6</v>
       </c>
     </row>
     <row r="5">
@@ -11205,10 +11217,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>18.6</v>
+        <v>19</v>
       </c>
       <c r="E5" t="n">
-        <v>14.6</v>
+        <v>15.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gun ici veri yenilemesi (BIST 100 yillik getiri, USD endeksi)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1,38 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kapak_Ozet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Katalog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Performans" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Performans_Ek_Kriter" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Fiyat_Serisi" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Portfoy_Dagilimi" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Getiri_Analizi_Detay" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Yillik_Getiri_Karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Temettu_Verimi" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Piyasa_Senaryolari" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Makro_Gostergeler" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Degerleme_CDS_MSCI" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bist_Yillik_Getiriler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer_PE_Karsilastirma" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Metinleri" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sabit_Metinler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Avantajlari_Maddeler" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi_Bireysel_Fon_Listesi" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi_ANZ_Tablosu" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ekip" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ekip_Organizasyon" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ata_Fonlari_Performans_Ozet" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ata_Fonlari_Performans_Ozet_YBB" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatirim_100TL_Dagilim" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatirim_100TL_Maddeler" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Kapak_Ozet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fon_Katalog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Fon_Performans" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Fon_Performans_Ek_Kriter" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Fon_Fiyat_Serisi" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Fon_Portfoy_Dagilimi" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Fon_Getiri_Analizi_Detay" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Fon_Yillik_Getiri_Karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Fon_Temettu_Verimi" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Piyasa_Senaryolari" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Makro_Gostergeler" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Degerleme_CDS_MSCI" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Bist_Yillik_Getiriler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Peer_PE_Karsilastirma" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Fon_Metinleri" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Sabit_Metinler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Fon_Avantajlari_Maddeler" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Vergi_Bireysel_Fon_Listesi" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Vergi_ANZ_Tablosu" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Ekip" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Ekip_Organizasyon" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Ata_Fonlari_Performans_Ozet" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Ata_Fonlari_Performans_Ozet_YBB" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Yatirim_100TL_Dagilim" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Yatirim_100TL_Maddeler" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3392,7 +3392,7 @@
         <v>2026</v>
       </c>
       <c r="B39" s="8" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Haftalik veri guncellemesi + Sayfa 24 Turkiye CDS otomatiklestirildi
Degerleme_CDS_MSCI'deki "Turkiye CDS" satiri artik Mete'nin elle
yeniledigi BBG_Weekly.xlsx'e degil, ANZ sayfasinin CDS mini-grafiginde
zaten kullanilan worldgovernmentbonds.com kaynagina bagli
(guncelle_degerleme_fk.py, haftalik_calistir.py). 07-27'den beri bayat
kalan 258 degeri, guncel 217,35'e (08-31) cekildi.
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1466,7 +1466,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>14128</v>
+        <v>14473</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>13000</v>
@@ -1490,7 +1490,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>47.92</v>
+        <v>48.12</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>54.7</v>
@@ -1514,7 +1514,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>56.07</v>
+        <v>56.03</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>63.4</v>
@@ -1538,7 +1538,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>7786</v>
+        <v>7674</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>7000</v>
@@ -1562,7 +1562,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>6468</v>
+        <v>6456</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>5800</v>
@@ -3036,7 +3036,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -3045,7 +3045,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>258</v>
+        <v>217.35</v>
       </c>
     </row>
     <row r="6">
@@ -4397,7 +4397,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B2" s="8" t="n">
@@ -5113,7 +5113,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>25</v>
+        <v>21.9</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5131,7 +5131,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>24.4</v>
+        <v>21.1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>37.2</v>
+        <v>33.5</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>53</v>
+        <v>49.7</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5185,7 +5185,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>35.1</v>
+        <v>29.8</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5203,7 +5203,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>38.6</v>
+        <v>32.9</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>43</v>
+        <v>40.6</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5239,7 +5239,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>50.1</v>
+        <v>50</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5257,7 +5257,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>44.1</v>
+        <v>43.9</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5275,7 +5275,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>47.1</v>
+        <v>47</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5293,7 +5293,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>37.5</v>
+        <v>33.1</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5329,7 +5329,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>32.6</v>
+        <v>31.3</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5347,7 +5347,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>52.5</v>
+        <v>53.1</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>54.8</v>
+        <v>51.9</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>37.4</v>
+        <v>40.3</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5401,7 +5401,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>22.6</v>
+        <v>22.4</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5419,7 +5419,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>17.3</v>
+        <v>17.5</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -5516,7 +5516,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>22.4</v>
+        <v>22.9</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5534,7 +5534,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>19.1</v>
+        <v>19.3</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5552,7 +5552,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>42.2</v>
+        <v>44.2</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5570,7 +5570,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>27.4</v>
+        <v>30.8</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5588,7 +5588,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>23.8</v>
+        <v>23.4</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5606,7 +5606,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>31.2</v>
+        <v>30.8</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5624,7 +5624,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>41.9</v>
+        <v>42.8</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5642,7 +5642,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>30.4</v>
+        <v>31.6</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5660,7 +5660,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>34</v>
+        <v>33.9</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5678,7 +5678,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>34.7</v>
+        <v>36.4</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5696,7 +5696,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>27.2</v>
+        <v>28.1</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5714,7 +5714,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>12.1</v>
+        <v>10.9</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5768,7 +5768,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>21.3</v>
+        <v>24.5</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5786,7 +5786,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>11.7</v>
+        <v>12.2</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5804,7 +5804,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>29</v>
+        <v>29.9</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5822,7 +5822,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>24</v>
+        <v>24.9</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -6791,7 +6791,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6805,16 +6805,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="E2" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6828,7 +6828,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
       <c r="E3" t="n">
         <v>10.8</v>
@@ -6837,7 +6837,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6851,16 +6851,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>18.1</v>
+        <v>18.2</v>
       </c>
       <c r="E4" t="n">
-        <v>20.2</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6874,16 +6874,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>44.1</v>
+        <v>43.9</v>
       </c>
       <c r="E5" t="n">
-        <v>45.6</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6897,16 +6897,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>24.9</v>
       </c>
       <c r="E6" t="n">
-        <v>26.1</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6920,16 +6920,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>5.8</v>
+        <v>11.4</v>
       </c>
       <c r="E7" t="n">
-        <v>3.1</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6943,16 +6943,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>8.9</v>
+        <v>11.8</v>
       </c>
       <c r="E8" t="n">
-        <v>3.8</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6966,16 +6966,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8.5</v>
+        <v>10.4</v>
       </c>
       <c r="E9" t="n">
-        <v>3.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6989,16 +6989,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>43</v>
+        <v>40.6</v>
       </c>
       <c r="E10" t="n">
-        <v>35.1</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -7012,16 +7012,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>34.7</v>
+        <v>36.4</v>
       </c>
       <c r="E11" t="n">
-        <v>30.4</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -7035,16 +7035,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.7</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -7058,16 +7058,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="E13" t="n">
-        <v>6.1</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7081,16 +7081,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>11.4</v>
+        <v>11.1</v>
       </c>
       <c r="E14" t="n">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -7104,16 +7104,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>37.5</v>
+        <v>33.1</v>
       </c>
       <c r="E15" t="n">
-        <v>40.6</v>
+        <v>34.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7127,16 +7127,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>31.2</v>
+        <v>30.8</v>
       </c>
       <c r="E16" t="n">
-        <v>32.8</v>
+        <v>31.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -7150,16 +7150,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1.3</v>
+        <v>12.4</v>
       </c>
       <c r="E17" t="n">
-        <v>7.9</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7173,16 +7173,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>7.2</v>
+        <v>5.4</v>
       </c>
       <c r="E18" t="n">
-        <v>18.1</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7196,16 +7196,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>40.7</v>
+        <v>37.4</v>
       </c>
       <c r="E19" t="n">
-        <v>43.1</v>
+        <v>41.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7222,13 +7222,13 @@
         <v>61</v>
       </c>
       <c r="E20" t="n">
-        <v>54.8</v>
+        <v>50.4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7242,16 +7242,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>41.9</v>
+        <v>42.8</v>
       </c>
       <c r="E21" t="n">
-        <v>53.2</v>
+        <v>50.6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7265,16 +7265,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>5.3</v>
+        <v>6.8</v>
       </c>
       <c r="E22" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7288,16 +7288,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>12.4</v>
+        <v>10.4</v>
       </c>
       <c r="E23" t="n">
-        <v>10.7</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7311,16 +7311,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8.300000000000001</v>
+        <v>7.8</v>
       </c>
       <c r="E24" t="n">
-        <v>20.7</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7334,16 +7334,16 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>32.6</v>
+        <v>31.3</v>
       </c>
       <c r="E25" t="n">
-        <v>45.7</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7357,16 +7357,16 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>23.8</v>
+        <v>23.4</v>
       </c>
       <c r="E26" t="n">
-        <v>39.6</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7380,16 +7380,16 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>7.5</v>
+        <v>17.7</v>
       </c>
       <c r="E27" t="n">
-        <v>6.3</v>
+        <v>18.2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7403,16 +7403,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1.8</v>
+        <v>3.5</v>
       </c>
       <c r="E28" t="n">
-        <v>-1</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7426,16 +7426,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>8.5</v>
+        <v>10.1</v>
       </c>
       <c r="E29" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7449,16 +7449,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>52.5</v>
+        <v>53.1</v>
       </c>
       <c r="E30" t="n">
-        <v>36.8</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7472,16 +7472,16 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>27.4</v>
+        <v>30.8</v>
       </c>
       <c r="E31" t="n">
-        <v>20</v>
+        <v>23.2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7495,16 +7495,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2.5</v>
+        <v>5.9</v>
       </c>
       <c r="E32" t="n">
-        <v>4.5</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7518,16 +7518,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2.9</v>
+        <v>6.2</v>
       </c>
       <c r="E33" t="n">
-        <v>7.6</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7541,16 +7541,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>-2.1</v>
+        <v>-1.6</v>
       </c>
       <c r="E34" t="n">
-        <v>5.8</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7564,16 +7564,16 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>24.4</v>
+        <v>21.1</v>
       </c>
       <c r="E35" t="n">
-        <v>38.6</v>
+        <v>32.9</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7587,16 +7587,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>19.1</v>
+        <v>19.3</v>
       </c>
       <c r="E36" t="n">
-        <v>34</v>
+        <v>33.9</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7610,16 +7610,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4775.2</v>
+        <v>4783.7</v>
       </c>
       <c r="E37" t="n">
-        <v>5340.2</v>
+        <v>5336.2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7633,16 +7633,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>4.8</v>
+        <v>7.5</v>
       </c>
       <c r="E38" t="n">
-        <v>3.1</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7656,16 +7656,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>3.2</v>
+        <v>6.8</v>
       </c>
       <c r="E39" t="n">
-        <v>3.8</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7679,16 +7679,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>-0.3</v>
+        <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>3.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7702,16 +7702,16 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>25</v>
+        <v>21.9</v>
       </c>
       <c r="E41" t="n">
-        <v>35.1</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7725,16 +7725,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>22.4</v>
+        <v>22.9</v>
       </c>
       <c r="E42" t="n">
-        <v>30.4</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7748,16 +7748,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>6264.8</v>
+        <v>6292.1</v>
       </c>
       <c r="E43" t="n">
-        <v>2809.4</v>
+        <v>2835.2</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7771,16 +7771,16 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>109.5</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E44" t="n">
-        <v>99.09999999999999</v>
+        <v>97.3</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7794,16 +7794,16 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1239.1</v>
+        <v>1248.9</v>
       </c>
       <c r="E45" t="n">
-        <v>1035.8</v>
+        <v>1035.2</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7817,16 +7817,16 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4.9</v>
+        <v>10.2</v>
       </c>
       <c r="E46" t="n">
-        <v>6.5</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7840,16 +7840,16 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>6.7</v>
+        <v>10.5</v>
       </c>
       <c r="E47" t="n">
-        <v>12.8</v>
+        <v>16.4</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7863,16 +7863,16 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>18.7</v>
+        <v>23.3</v>
       </c>
       <c r="E48" t="n">
-        <v>28.6</v>
+        <v>33.5</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7886,16 +7886,16 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>53</v>
+        <v>49.7</v>
       </c>
       <c r="E49" t="n">
-        <v>63</v>
+        <v>58.8</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7909,16 +7909,16 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>42.2</v>
+        <v>44.2</v>
       </c>
       <c r="E50" t="n">
-        <v>55.7</v>
+        <v>59.1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -7932,16 +7932,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>12.6</v>
+        <v>12.9</v>
       </c>
       <c r="E51" t="n">
-        <v>12.7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -7955,16 +7955,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>6.2</v>
+        <v>3.3</v>
       </c>
       <c r="E52" t="n">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -7978,16 +7978,16 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-2.7</v>
+        <v>-6.5</v>
       </c>
       <c r="E53" t="n">
-        <v>0.6</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -8001,7 +8001,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>54.8</v>
+        <v>51.9</v>
       </c>
       <c r="E54" t="n">
         <v>57.1</v>
@@ -8010,7 +8010,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -8024,16 +8024,16 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>12.1</v>
+        <v>10.9</v>
       </c>
       <c r="E55" t="n">
-        <v>15.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -8047,13 +8047,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>5.8</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -8067,13 +8067,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>6.7</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -8087,13 +8087,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>19.6</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -8107,13 +8107,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>37.4</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -8127,13 +8127,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>21.3</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -8147,16 +8147,16 @@
         </is>
       </c>
       <c r="D61" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E61" t="n">
         <v>3.4</v>
-      </c>
-      <c r="E61" t="n">
-        <v>3.3</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -8170,16 +8170,16 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>11.1</v>
+        <v>10.6</v>
       </c>
       <c r="E62" t="n">
-        <v>10.4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -8202,7 +8202,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -8216,16 +8216,16 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>50.1</v>
+        <v>50</v>
       </c>
       <c r="E64" t="n">
-        <v>47.1</v>
+        <v>47</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -8239,16 +8239,16 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>29</v>
+        <v>29.9</v>
       </c>
       <c r="E65" t="n">
-        <v>27.2</v>
+        <v>28.1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -8271,7 +8271,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -8285,7 +8285,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>6.5</v>
+        <v>7.1</v>
       </c>
       <c r="E67" t="n">
         <v>0.6</v>
@@ -8294,7 +8294,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -8308,7 +8308,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>9.699999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="E68" t="n">
         <v>1.2</v>
@@ -8317,7 +8317,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -8331,7 +8331,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>22.6</v>
+        <v>22.4</v>
       </c>
       <c r="E69" t="n">
         <v>2.1</v>
@@ -8340,7 +8340,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -8354,7 +8354,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="E70" t="n">
         <v>1.4</v>
@@ -8363,7 +8363,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -8377,13 +8377,13 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -8397,13 +8397,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>10.8</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -8480,7 +8480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8505,7 +8505,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8524,13 +8524,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8549,13 +8549,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>9.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8574,13 +8574,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>17.3</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8599,13 +8599,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>11.7</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8624,13 +8624,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8649,13 +8649,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10.4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8680,7 +8680,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8699,13 +8699,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>47.1</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -8724,13 +8724,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>27.2</v>
+        <v>28.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -8749,13 +8749,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -8774,13 +8774,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>7.5</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -8799,13 +8799,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>9.6</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -8824,13 +8824,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>39.8</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -8849,13 +8849,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>31.4</v>
+        <v>31.8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -8874,13 +8874,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>-7.1</v>
+        <v>-6.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -8899,13 +8899,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>3.4</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -8924,13 +8924,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>6.8</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -8949,13 +8949,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>41.9</v>
+        <v>33.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -8974,13 +8974,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>35.3</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -8999,13 +8999,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9024,13 +9024,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>16.4</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9049,13 +9049,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>30.6</v>
+        <v>30.7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9074,13 +9074,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>38.4</v>
+        <v>41.1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9099,13 +9099,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>28.8</v>
+        <v>30.5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -9124,13 +9124,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>-4.4</v>
+        <v>-9.1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -9149,13 +9149,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>21.4</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -9174,13 +9174,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>66.3</v>
+        <v>61.1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -9199,13 +9199,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>85.09999999999999</v>
+        <v>67.8</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -9224,13 +9224,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>98.40000000000001</v>
+        <v>87.90000000000001</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -9249,13 +9249,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>3.44</v>
+        <v>3.43</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -9274,13 +9274,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>10.77</v>
+        <v>11.13</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -9299,13 +9299,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>22.49</v>
+        <v>22.56</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -9324,13 +9324,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>50.25</v>
+        <v>50.12</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -9349,7 +9349,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>29.17</v>
+        <v>30.18</v>
       </c>
     </row>
   </sheetData>
@@ -9497,7 +9497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9511,13 +9511,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>9.24</v>
+        <v>10.21</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9531,13 +9531,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>10.89</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9551,13 +9551,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.09</v>
+        <v>3.43</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9567,17 +9567,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Kamu Kira Sertifikası (TL)</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.33</v>
+        <v>5.32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9587,17 +9587,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Kamu Kira Sertifikası (TL)</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.71</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9607,17 +9607,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2.48</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9627,17 +9627,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Takasbank Para Piyasası</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.68</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9647,17 +9647,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Takasbank Para Piyasası</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>48.48</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -9667,17 +9667,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3.21</v>
+        <v>36.57</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -9687,17 +9687,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>19.86</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -9707,22 +9707,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.03</v>
+        <v>25.78</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AAS</t>
+          <t>AAL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -9731,13 +9731,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.66</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -9747,17 +9747,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>39.86</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -9767,37 +9767,37 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>59.48</v>
+        <v>69.31999999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>AAV</t>
+          <t>AAS</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>92.27</v>
+        <v>30.31</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9807,17 +9807,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3.99</v>
+        <v>86.81999999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -9827,37 +9827,37 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3.74</v>
+        <v>9.65</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AED</t>
+          <t>AAV</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Devlet Tahvili</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>5.42</v>
+        <v>3.53</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9867,17 +9867,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Devlet Tahvili</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3.33</v>
+        <v>10.39</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9887,17 +9887,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>55.41</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9907,17 +9907,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1.05</v>
+        <v>55.21</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9927,17 +9927,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>3.09</v>
+        <v>22.85</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9947,37 +9947,37 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>18.83</v>
+        <v>8.359999999999999</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AED</t>
+          <t>ANZ</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Kamu Dış Borçlanma Araçları</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>12.87</v>
+        <v>90.59</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9987,17 +9987,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Vadeli Mevduat (Döviz)</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1.88</v>
+        <v>7.39</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -10007,17 +10007,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Özel Sektör Dış Borçlanma Araçları</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>98.12</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -10031,13 +10031,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>85.7</v>
+        <v>88.25</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -10051,13 +10051,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.92</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -10067,57 +10067,57 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2.21</v>
+        <v>10.79</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>AYA</t>
+          <t>DGH</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.16</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>AYA</t>
+          <t>DGH</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>11.01</v>
+        <v>6.28</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -10127,17 +10127,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1.02</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -10147,17 +10147,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.8100000000000001</v>
+        <v>21.58</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -10167,17 +10167,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>22.39</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -10187,37 +10187,37 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1.02</v>
+        <v>69.3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DGH</t>
+          <t>JET</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>74.76000000000001</v>
+        <v>23.47</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -10227,17 +10227,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>23.42</v>
+        <v>3.66</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -10247,17 +10247,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>2.75</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -10267,17 +10267,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.86</v>
+        <v>66.66</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -10287,37 +10287,37 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>67.17</v>
+        <v>6.07</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>JET</t>
+          <t>PKF</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>5.8</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -10331,13 +10331,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3.24</v>
+        <v>3.27</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -10351,13 +10351,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>94.68000000000001</v>
+        <v>80.09</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -10371,13 +10371,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>2.08</v>
+        <v>7.84</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10391,13 +10391,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>78.22</v>
+        <v>81.68000000000001</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -10411,13 +10411,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>21.78</v>
+        <v>18.32</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -10431,13 +10431,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>22.62</v>
+        <v>21.11</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -10451,13 +10451,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.52</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -10471,13 +10471,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>64.47</v>
+        <v>65.97</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -10491,13 +10491,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>12.39</v>
+        <v>12.57</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -10511,13 +10511,13 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>88.77</v>
+        <v>87.91</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -10531,13 +10531,13 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>11.23</v>
+        <v>12.09</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10551,13 +10551,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1.48</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -10571,13 +10571,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>14.71</v>
+        <v>16.71</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -10591,13 +10591,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1.17</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -10611,13 +10611,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -10631,13 +10631,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>71.8</v>
+        <v>67.43000000000001</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -10651,13 +10651,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>10.81</v>
+        <v>10.64</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -10671,13 +10671,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>31.25</v>
+        <v>31.08</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -10691,13 +10691,13 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -10711,13 +10711,13 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>67.45999999999999</v>
+        <v>67.87</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -10731,7 +10731,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.48</v>
+        <v>0.54</v>
       </c>
     </row>
   </sheetData>
@@ -10841,22 +10841,22 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>25</v>
+        <v>21.9</v>
       </c>
       <c r="E2" t="n">
-        <v>109.5</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>1239.1</v>
+        <v>1248.9</v>
       </c>
       <c r="G2" t="n">
-        <v>6264.8</v>
+        <v>6292.1</v>
       </c>
       <c r="H2" t="n">
-        <v>28</v>
+        <v>25.9</v>
       </c>
       <c r="I2" t="n">
-        <v>68</v>
+        <v>68.3</v>
       </c>
       <c r="J2" t="n">
         <v>35.2</v>
@@ -10884,25 +10884,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>35.1</v>
+        <v>29.8</v>
       </c>
       <c r="E3" t="n">
-        <v>99.09999999999999</v>
+        <v>97.3</v>
       </c>
       <c r="F3" t="n">
-        <v>1035.8</v>
+        <v>1035.2</v>
       </c>
       <c r="G3" t="n">
-        <v>2809.4</v>
+        <v>2835.2</v>
       </c>
       <c r="H3" t="n">
-        <v>25.8</v>
+        <v>25.4</v>
       </c>
       <c r="I3" t="n">
         <v>62.6</v>
       </c>
       <c r="J3" t="n">
-        <v>27.7</v>
+        <v>27.8</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -10927,25 +10927,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-10.1</v>
+        <v>-7.9</v>
       </c>
       <c r="E4" t="n">
-        <v>10.4</v>
+        <v>2.1</v>
       </c>
       <c r="F4" t="n">
-        <v>203.3</v>
+        <v>213.7</v>
       </c>
       <c r="G4" t="n">
-        <v>3455.4</v>
+        <v>3456.9</v>
       </c>
       <c r="H4" t="n">
-        <v>2.2</v>
+        <v>0.5</v>
       </c>
       <c r="I4" t="n">
-        <v>5.4</v>
+        <v>5.7</v>
       </c>
       <c r="J4" t="n">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -10970,22 +10970,22 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>27.7</v>
+        <v>24.6</v>
       </c>
       <c r="E5" t="n">
-        <v>121.4</v>
+        <v>110.7</v>
       </c>
       <c r="F5" t="n">
-        <v>1368.7</v>
+        <v>1379.4</v>
       </c>
       <c r="G5" t="n">
-        <v>7985.7</v>
+        <v>8020.4</v>
       </c>
       <c r="H5" t="n">
-        <v>30.3</v>
+        <v>28.2</v>
       </c>
       <c r="I5" t="n">
-        <v>71.2</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="J5" t="n">
         <v>37.6</v>
@@ -11013,25 +11013,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>35.1</v>
+        <v>29.8</v>
       </c>
       <c r="E6" t="n">
-        <v>99.09999999999999</v>
+        <v>97.3</v>
       </c>
       <c r="F6" t="n">
-        <v>1035.8</v>
+        <v>1035.2</v>
       </c>
       <c r="G6" t="n">
-        <v>2809.4</v>
+        <v>2835.2</v>
       </c>
       <c r="H6" t="n">
-        <v>25.8</v>
+        <v>25.4</v>
       </c>
       <c r="I6" t="n">
         <v>62.6</v>
       </c>
       <c r="J6" t="n">
-        <v>27.7</v>
+        <v>27.8</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -11056,25 +11056,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-7.4</v>
+        <v>-5.2</v>
       </c>
       <c r="E7" t="n">
-        <v>22.3</v>
+        <v>13.4</v>
       </c>
       <c r="F7" t="n">
-        <v>332.9</v>
+        <v>344.2</v>
       </c>
       <c r="G7" t="n">
-        <v>5176.3</v>
+        <v>5185.2</v>
       </c>
       <c r="H7" t="n">
-        <v>4.5</v>
+        <v>2.8</v>
       </c>
       <c r="I7" t="n">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -11148,10 +11148,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>28</v>
+        <v>25.9</v>
       </c>
       <c r="E2" t="n">
-        <v>25.8</v>
+        <v>25.4</v>
       </c>
     </row>
     <row r="3">
@@ -11171,10 +11171,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5.9</v>
+        <v>3.3</v>
       </c>
       <c r="E3" t="n">
-        <v>4.2</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="4">
@@ -11194,7 +11194,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>68</v>
+        <v>68.3</v>
       </c>
       <c r="E4" t="n">
         <v>62.6</v>
@@ -11217,10 +11217,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>19</v>
+        <v>18.6</v>
       </c>
       <c r="E5" t="n">
-        <v>15.1</v>
+        <v>14.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sunumdaki yazim hatalari duzeltildi
Ata Grubu tanitim metni, vergi metni, yasal uyari, AAV/JET fon
aciklamalari, ekip unvani ve yillik getiri baslik etiketlerindeki
yazim/tutarlilik hatalari giderildi.
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1,38 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Kapak_Ozet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Fon_Katalog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Fon_Performans" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Fon_Performans_Ek_Kriter" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Fon_Fiyat_Serisi" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Fon_Portfoy_Dagilimi" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Fon_Getiri_Analizi_Detay" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Fon_Yillik_Getiri_Karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Fon_Temettu_Verimi" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Piyasa_Senaryolari" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Makro_Gostergeler" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Degerleme_CDS_MSCI" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Bist_Yillik_Getiriler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Peer_PE_Karsilastirma" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Fon_Metinleri" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Sabit_Metinler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Fon_Avantajlari_Maddeler" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Vergi_Bireysel_Fon_Listesi" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Vergi_ANZ_Tablosu" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Ekip" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Ekip_Organizasyon" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Ata_Fonlari_Performans_Ozet" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Ata_Fonlari_Performans_Ozet_YBB" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Yatirim_100TL_Dagilim" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Yatirim_100TL_Maddeler" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kapak_Ozet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Katalog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Performans" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Performans_Ek_Kriter" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Fiyat_Serisi" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Portfoy_Dagilimi" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Getiri_Analizi_Detay" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Yillik_Getiri_Karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Temettu_Verimi" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Piyasa_Senaryolari" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Makro_Gostergeler" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Degerleme_CDS_MSCI" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bist_Yillik_Getiriler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer_PE_Karsilastirma" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Metinleri" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sabit_Metinler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Avantajlari_Maddeler" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi_Bireysel_Fon_Listesi" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi_ANZ_Tablosu" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ekip" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ekip_Organizasyon" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ata_Fonlari_Performans_Ozet" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ata_Fonlari_Performans_Ozet_YBB" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatirim_100TL_Dagilim" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatirim_100TL_Maddeler" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>48.12</v>
+        <v>48.22</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>54.7</v>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>56.03</v>
+        <v>55.92</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>63.4</v>
@@ -3392,7 +3392,7 @@
         <v>2026</v>
       </c>
       <c r="B39" s="8" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -3654,7 +3654,7 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>Fon, ağırlıklı BIST100'de işlem gören ve kar büyüme potansiyeli olan 30-35 şirkete yatırım yapar. Fon yönetiminde aktif yönetim modeli uygulanır. Fon'un karşılaştırma ölçütü BIST-100 Getiri Endeksi'dir. Stopaj oranı %0'dır.</t>
+          <t>Fon, ağırlıklı BIST100'de işlem gören ve kâr büyüme potansiyeli olan 30-35 şirkete yatırım yapar. Fon yönetiminde aktif yönetim modeli uygulanır. Fon'un karşılaştırma ölçütü BIST-100 Getiri Endeksi'dir. Stopaj oranı %0'dır.</t>
         </is>
       </c>
     </row>
@@ -3750,7 +3750,7 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Ata Portföy Havacılık ve Savunma Teknolojileri Değişken Fon; havacılık, uzay ve savunma alanlarında gelişen teknolojiler, artan stratejik işbirlikleri ve yükselen kamu harcamaları ile ortaya çıkan uzun vadeli küresel büyüme potansiyeline yatırım imkanı sunmayı hedefler. Fon, yerli ve yabancı havacılık, uzay ve savunma alanında faaliyet gösteren şirketlere yatırım yaparak bu sektörlerdeki teknolojik gelişmeler ve ekonomik büyümeye paydaş olma imkanı sunar. Türkiye, Amerika, Avrupa ve Asya şirketlerinden oluşturulan fon portföyü küresel çeşitlendirme imkanı sunmaktadır. Karşılaştırma ölçütü %65 Nasdaq US Benchmark Aerospace and Defense Total Return Index + %35 BIST Teknoloji Ağırlık Sınırlamalı Getiri Endeksi olarak belirlenmiştir. %17,5 stopaja tabidir.</t>
+          <t>Ata Portföy Havacılık ve Savunma Teknolojileri Değişken Fon; havacılık, uzay ve savunma alanlarında gelişen teknolojiler, artan stratejik işbirlikleri ve yükselen kamu harcamaları ile ortaya çıkan uzun vadeli küresel büyüme potansiyeline yatırım imkânı sunmayı hedefler. Fon, yerli ve yabancı havacılık, uzay ve savunma alanında faaliyet gösteren şirketlere yatırım yaparak bu sektörlerdeki teknolojik gelişmeler ve ekonomik büyümeye paydaş olma imkânı sunar. Türkiye, Amerika, Avrupa ve Asya şirketlerinden oluşturulan fon portföyü küresel çeşitlendirme imkânı sunmaktadır. Karşılaştırma ölçütü %65 Nasdaq US Benchmark Aerospace and Defense Total Return Index + %35 BIST Teknoloji Ağırlık Sınırlamalı Getiri Endeksi olarak belirlenmiştir. %17,5 stopaja tabidir.</t>
         </is>
       </c>
     </row>
@@ -3842,7 +3842,7 @@
       <c r="B3" s="14" t="inlineStr">
         <is>
           <t>Ata Holding'in kökleri, Atatürk Barajını yapan Ata İnşaat'a uzanır. Güneydoğu Anadolu Projesi (GAP) içinde yer alan Atatürk Barajı Hidroelektrik Santralini tamamlayan konsorsiyumun üç üyesinden biri olan Seri İnşaat, Grubumuz kurucu Sayın Ertuğrul Kurdoğlu'nun 1969 yılında kurduğu ilk mühendislik şirketidir.
-Ata Grubu'nun faaliyet alanı zaman içinde finans, teknoloji, gıda, lojistik, gayrimenkul geliştirme, yapı malzemeleri, moda, turizm ve dış ticarete evrildi. Finans alanında ATA, gıda alanında TAB markasıyla önce çıkan Ata Holding, Türkiye başta olmak üzere pek çok ülkede Burger King master "franchise" sahibidir.
+Ata Grubu'nun faaliyet alanı zaman içinde finans, teknoloji, gıda, lojistik, gayrimenkul geliştirme, yapı malzemeleri, moda, turizm ve dış ticarete evrildi. Finans alanında ATA, gıda alanında TAB markasıyla öne çıkan Ata Holding, Türkiye başta olmak üzere pek çok ülkede Burger King master "franchise" sahibidir.
 Dört kıta ve sekiz ülkede 30'dan fazla şirketle faaliyet gösteren Ata Holding'in yaygın portföy yapısı, risklere karşı koruma sağlamaktadır. Bu kapsamda Grubumuz 30.000'den fazla personele istihdam olanağı sunmaktadır.</t>
         </is>
       </c>
@@ -3915,7 +3915,7 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>Fonlarda stopaj oranı  9 Temmuz 2025 itibarı ile %15'ten %17,5'a çıkartıldı.</t>
+          <t>Fonlarda stopaj oranı 9 Temmuz 2025 itibarı ile %15'ten %17,5'a çıkartıldı.</t>
         </is>
       </c>
     </row>
@@ -4119,7 +4119,7 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Bu sunumda yer alan bilgiler Ata Portföy tarafından bilgilendirme amacıyla hazırlanmıştır. Yatırım bilgi, yorum ve tavsiyeleri yatırım danışmanlığı kapsamında değildir. Yatırım danışmanlığı hizmeti; aracı kurumlar, portföy yönetim şirketleri, mevduat kabul etmeyen bankalar ile müşteri arasında imzalanacak yatırım danışmanlığı sözleşmesi çerçevesinde sunulmaktadır. Burada yer alan yorum ve tavsiyeler, yorum ve tavsiyede bulunanların kişisel görüşlerine dayanmaktadır. Bu görüşlere ilişkin bilgiler güvenilirliğine inanılan kaynaklardan elde edilmiş olup, Ata Portföy bu bilgilerin doğruluğu hakkında garanti vermemektedir. Bu görüşler, mali durumunuz ile risk ve getiri tercihlerinize uygun olmayabilir. Bu nedenle, sadece burada yer alan bilgilere dayanılarak yatırım kararı verilmesi beklentilerinize uygun sonuçlar doğurmayabilir. Bu durumda, ortaya çıkabilecek sonuçlardan dolayı Ata Portföy sorumluluk kabul etmez. Ata Portföy, hiçbir şekil ve surette ön ihbara ve/veya ihtara gerek verebileceği herhangi bir zarardan sorumlu tutulamaz. Bu e-postanın virüs içermemesi için alınması gereken tedbirler alınmıştır. İşbu e-posta ve eklerinin kullanımından kaynaklı zarar veya kayıplardan sorumlu olmadığımızı kullanmadan önce virüs kontrol programlarınızı uygulamanızı tavsiye ederiz.</t>
+          <t>Bu sunumda yer alan bilgiler Ata Portföy tarafından bilgilendirme amacıyla hazırlanmıştır. Yatırım bilgi, yorum ve tavsiyeleri yatırım danışmanlığı kapsamında değildir. Yatırım danışmanlığı hizmeti; aracı kurumlar, portföy yönetim şirketleri, mevduat kabul etmeyen bankalar ile müşteri arasında imzalanacak yatırım danışmanlığı sözleşmesi çerçevesinde sunulmaktadır. Burada yer alan yorum ve tavsiyeler, yorum ve tavsiyede bulunanların kişisel görüşlerine dayanmaktadır. Bu görüşlere ilişkin bilgiler güvenilirliğine inanılan kaynaklardan elde edilmiş olup, Ata Portföy bu bilgilerin doğruluğu hakkında garanti vermemektedir. Bu görüşler, mali durumunuz ile risk ve getiri tercihlerinize uygun olmayabilir. Bu nedenle, sadece burada yer alan bilgilere dayanılarak yatırım kararı verilmesi beklentilerinize uygun sonuçlar doğurmayabilir. Bu durumda, ortaya çıkabilecek sonuçlardan dolayı Ata Portföy sorumluluk kabul etmez. Ata Portföy, önceden ihbar ve/veya ihtarda bulunmaksızın hiçbir şekil ve surette doğabilecek herhangi bir zarardan sorumlu tutulamaz. Bu e-postanın virüs içermemesi için alınması gereken tedbirler alınmıştır. İşbu e-posta ve eklerinin kullanımından kaynaklı zarar veya kayıplardan sorumlu olmadığımızı kullanmadan önce virüs kontrol programlarınızı uygulamanızı tavsiye ederiz.</t>
         </is>
       </c>
     </row>
@@ -4714,7 +4714,7 @@
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>CEO, Board Member</t>
+          <t>CEO, Yönetim Kurulu Üyesi</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>51.9</v>
+        <v>54.6</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5714,7 +5714,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10.9</v>
+        <v>12.9</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -7932,7 +7932,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>12.9</v>
+        <v>14.9</v>
       </c>
       <c r="E51" t="n">
         <v>14</v>
@@ -7955,7 +7955,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>3.3</v>
+        <v>5.1</v>
       </c>
       <c r="E52" t="n">
         <v>6.3</v>
@@ -7978,7 +7978,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-6.5</v>
+        <v>-4.9</v>
       </c>
       <c r="E53" t="n">
         <v>-2.5</v>
@@ -8001,7 +8001,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>51.9</v>
+        <v>54.6</v>
       </c>
       <c r="E54" t="n">
         <v>57.1</v>
@@ -8024,7 +8024,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>10.9</v>
+        <v>12.9</v>
       </c>
       <c r="E55" t="n">
         <v>16.5</v>
@@ -11139,7 +11139,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Son 3 Yil</t>
+          <t>Son 3 Yıl</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -11162,7 +11162,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Son 3 Yil</t>
+          <t>Son 3 Yıl</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11185,7 +11185,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Son 5 Yil</t>
+          <t>Son 5 Yıl</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -11208,7 +11208,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Son 5 Yil</t>
+          <t>Son 5 Yıl</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">

</xml_diff>

<commit_message>
Haftalik veri guncellemesi + Sayfa 11 AAV yillik getiri grafikleri duzeltildi
Fon_Yillik_Getiri_Karsilastirma sayfasindaki Donem degerleri ("Son 3/5 Yil",
noktali i) FonSayfalari.tsx'in aradigi "Son 3/5 Yıl" (noktasiz ı) ile
eslesmiyordu, bu yuzden Sayfa 11 basliktan sonra bos gorunuyordu.
guncelle_fon_getirileri.py ve mevcut Veri_Kaynagi.xlsx satirlari duzeltildi.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1,38 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kapak_Ozet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Katalog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Performans" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Performans_Ek_Kriter" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Fiyat_Serisi" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Portfoy_Dagilimi" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Getiri_Analizi_Detay" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Yillik_Getiri_Karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Temettu_Verimi" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Piyasa_Senaryolari" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Makro_Gostergeler" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Degerleme_CDS_MSCI" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bist_Yillik_Getiriler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer_PE_Karsilastirma" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Metinleri" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sabit_Metinler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Avantajlari_Maddeler" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi_Bireysel_Fon_Listesi" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi_ANZ_Tablosu" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ekip" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ekip_Organizasyon" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ata_Fonlari_Performans_Ozet" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ata_Fonlari_Performans_Ozet_YBB" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatirim_100TL_Dagilim" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatirim_100TL_Maddeler" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Kapak_Ozet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fon_Katalog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Fon_Performans" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Fon_Performans_Ek_Kriter" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Fon_Fiyat_Serisi" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Fon_Portfoy_Dagilimi" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Fon_Getiri_Analizi_Detay" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Fon_Yillik_Getiri_Karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Fon_Temettu_Verimi" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Piyasa_Senaryolari" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Makro_Gostergeler" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Degerleme_CDS_MSCI" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Bist_Yillik_Getiriler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Peer_PE_Karsilastirma" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Fon_Metinleri" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Sabit_Metinler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Fon_Avantajlari_Maddeler" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Vergi_Bireysel_Fon_Listesi" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Vergi_ANZ_Tablosu" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Ekip" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Ekip_Organizasyon" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Ata_Fonlari_Performans_Ozet" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Ata_Fonlari_Performans_Ozet_YBB" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Yatirim_100TL_Dagilim" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Yatirim_100TL_Maddeler" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1466,7 +1466,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>14473</v>
+        <v>14229</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>13000</v>
@@ -1490,7 +1490,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>48.22</v>
+        <v>48.28</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>54.7</v>
@@ -1514,7 +1514,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>55.92</v>
+        <v>56.11</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>63.4</v>
@@ -1538,7 +1538,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>7674</v>
+        <v>7712</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>7000</v>
@@ -1562,7 +1562,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>6456</v>
+        <v>6369</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>5800</v>
@@ -2991,7 +2991,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -3000,13 +3000,13 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>10.95</v>
+        <v>10.81</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>17.72</v>
+        <v>15.23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -3030,13 +3030,13 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>24.25</v>
+        <v>23.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -3045,7 +3045,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>217.35</v>
+        <v>218.68</v>
       </c>
     </row>
     <row r="6">
@@ -3392,7 +3392,7 @@
         <v>2026</v>
       </c>
       <c r="B39" s="8" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -3450,7 +3450,7 @@
     <row r="8">
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -3459,13 +3459,13 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>20.32</v>
+        <v>19.92</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -3474,13 +3474,13 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>18.06</v>
+        <v>16.92</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -3495,7 +3495,7 @@
     <row r="11">
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -3504,13 +3504,13 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>12.45</v>
+        <v>12.37</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -3519,13 +3519,13 @@
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>10.66</v>
+        <v>9.91</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -3534,13 +3534,13 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>9.74</v>
+        <v>9.140000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -3549,13 +3549,13 @@
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>9.390000000000001</v>
+        <v>9.359999999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -3564,13 +3564,13 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>8.59</v>
+        <v>9.449999999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -3579,13 +3579,13 @@
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>8.44</v>
+        <v>8.34</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -3594,7 +3594,7 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>6.69</v>
+        <v>7.18</v>
       </c>
     </row>
     <row r="18">
@@ -4397,7 +4397,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B2" s="8" t="n">
@@ -5113,7 +5113,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>21.9</v>
+        <v>21.5</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5131,7 +5131,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>21.1</v>
+        <v>18.7</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>33.5</v>
+        <v>30.9</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>49.7</v>
+        <v>40.2</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5185,7 +5185,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>29.8</v>
+        <v>26.4</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5203,7 +5203,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>32.9</v>
+        <v>33.4</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>40.6</v>
+        <v>37.9</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5239,7 +5239,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>50</v>
+        <v>49.8</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5257,7 +5257,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>43.9</v>
+        <v>43.6</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5275,7 +5275,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>47</v>
+        <v>46.9</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5293,7 +5293,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>33.1</v>
+        <v>36.2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5311,7 +5311,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>61</v>
+        <v>59.4</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5329,7 +5329,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>31.3</v>
+        <v>24.7</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5347,7 +5347,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>53.1</v>
+        <v>39.6</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>54.6</v>
+        <v>49.3</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>40.3</v>
+        <v>40.1</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5401,7 +5401,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>22.4</v>
+        <v>22.3</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5419,7 +5419,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5455,7 +5455,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>31.8</v>
+        <v>34.4</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -5516,7 +5516,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>22.9</v>
+        <v>20</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5534,7 +5534,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>19.3</v>
+        <v>15.4</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5552,7 +5552,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>44.2</v>
+        <v>34.4</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5570,7 +5570,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>30.8</v>
+        <v>27.1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5588,7 +5588,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>23.4</v>
+        <v>18.2</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5606,7 +5606,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>30.8</v>
+        <v>32.4</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5624,7 +5624,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>42.8</v>
+        <v>40.9</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5642,7 +5642,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>31.6</v>
+        <v>25.9</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5660,7 +5660,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>33.9</v>
+        <v>31.9</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5678,7 +5678,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>36.4</v>
+        <v>32.9</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5696,7 +5696,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>28.1</v>
+        <v>29</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5714,7 +5714,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>12.9</v>
+        <v>10.3</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13.7</v>
+        <v>13.9</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5768,7 +5768,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>24.5</v>
+        <v>24.8</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5786,7 +5786,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>12.2</v>
+        <v>12.6</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5804,7 +5804,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>29.9</v>
+        <v>30.9</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5822,7 +5822,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>24.9</v>
+        <v>25.7</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5840,7 +5840,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>19.9</v>
+        <v>24.8</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -6791,7 +6791,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6805,7 +6805,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2.1</v>
+        <v>3.3</v>
       </c>
       <c r="E2" t="n">
         <v>3.6</v>
@@ -6814,7 +6814,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6828,16 +6828,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>7.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>10.8</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6854,13 +6854,13 @@
         <v>18.2</v>
       </c>
       <c r="E4" t="n">
-        <v>20.5</v>
+        <v>20.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6874,16 +6874,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>43.9</v>
+        <v>43.6</v>
       </c>
       <c r="E5" t="n">
-        <v>45.7</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6897,16 +6897,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24.9</v>
+        <v>25.7</v>
       </c>
       <c r="E6" t="n">
-        <v>27.1</v>
+        <v>28.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6920,16 +6920,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>11.4</v>
+        <v>4.6</v>
       </c>
       <c r="E7" t="n">
-        <v>8.5</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6943,16 +6943,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>11.8</v>
+        <v>8.4</v>
       </c>
       <c r="E8" t="n">
-        <v>7.4</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6966,16 +6966,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>10.4</v>
+        <v>12.8</v>
       </c>
       <c r="E9" t="n">
-        <v>5.4</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6989,16 +6989,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>40.6</v>
+        <v>37.9</v>
       </c>
       <c r="E10" t="n">
-        <v>29.8</v>
+        <v>26.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -7012,16 +7012,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>36.4</v>
+        <v>32.9</v>
       </c>
       <c r="E11" t="n">
-        <v>31.6</v>
+        <v>25.9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -7035,16 +7035,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3.9</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -7058,16 +7058,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>7.1</v>
+        <v>8.5</v>
       </c>
       <c r="E13" t="n">
-        <v>5.5</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7081,16 +7081,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>11.1</v>
+        <v>15.3</v>
       </c>
       <c r="E14" t="n">
-        <v>8.5</v>
+        <v>14.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -7104,16 +7104,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>33.1</v>
+        <v>36.2</v>
       </c>
       <c r="E15" t="n">
-        <v>34.8</v>
+        <v>37.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7127,16 +7127,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>30.8</v>
+        <v>32.4</v>
       </c>
       <c r="E16" t="n">
-        <v>31.7</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -7150,16 +7150,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>12.4</v>
+        <v>0.6</v>
       </c>
       <c r="E17" t="n">
-        <v>6.1</v>
+        <v>-7.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7173,16 +7173,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>5.4</v>
+        <v>-1.3</v>
       </c>
       <c r="E18" t="n">
-        <v>11.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7196,16 +7196,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>37.4</v>
+        <v>42.8</v>
       </c>
       <c r="E19" t="n">
-        <v>41.4</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7219,16 +7219,16 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>61</v>
+        <v>59.4</v>
       </c>
       <c r="E20" t="n">
-        <v>50.4</v>
+        <v>39.9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7242,16 +7242,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>42.8</v>
+        <v>40.9</v>
       </c>
       <c r="E21" t="n">
-        <v>50.6</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7265,16 +7265,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>6.8</v>
+        <v>-3.8</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>-8.9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7288,16 +7288,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>10.4</v>
+        <v>4.2</v>
       </c>
       <c r="E23" t="n">
-        <v>6.2</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7311,16 +7311,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>7.8</v>
+        <v>3.5</v>
       </c>
       <c r="E24" t="n">
-        <v>17.6</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7334,16 +7334,16 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>31.3</v>
+        <v>24.7</v>
       </c>
       <c r="E25" t="n">
-        <v>40.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7357,16 +7357,16 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>23.4</v>
+        <v>18.2</v>
       </c>
       <c r="E26" t="n">
-        <v>37</v>
+        <v>28.8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7380,16 +7380,16 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>17.7</v>
+        <v>5.9</v>
       </c>
       <c r="E27" t="n">
-        <v>18.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7403,16 +7403,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3.5</v>
+        <v>1.1</v>
       </c>
       <c r="E28" t="n">
-        <v>-2.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7426,16 +7426,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>10.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E29" t="n">
-        <v>0.9</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7449,16 +7449,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>53.1</v>
+        <v>39.6</v>
       </c>
       <c r="E30" t="n">
-        <v>37.9</v>
+        <v>32.3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7472,16 +7472,16 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>30.8</v>
+        <v>27.1</v>
       </c>
       <c r="E31" t="n">
-        <v>23.2</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7495,16 +7495,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>5.9</v>
+        <v>-0.5</v>
       </c>
       <c r="E32" t="n">
-        <v>7.7</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7518,16 +7518,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>6.2</v>
+        <v>1.5</v>
       </c>
       <c r="E33" t="n">
-        <v>11.8</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7541,16 +7541,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>-1.6</v>
+        <v>2</v>
       </c>
       <c r="E34" t="n">
-        <v>6.9</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7564,16 +7564,16 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>21.1</v>
+        <v>18.7</v>
       </c>
       <c r="E35" t="n">
-        <v>32.9</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7587,16 +7587,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>19.3</v>
+        <v>15.4</v>
       </c>
       <c r="E36" t="n">
-        <v>33.9</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7610,16 +7610,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4783.7</v>
+        <v>4623.4</v>
       </c>
       <c r="E37" t="n">
-        <v>5336.2</v>
+        <v>5256.7</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7633,16 +7633,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>7.5</v>
+        <v>2.4</v>
       </c>
       <c r="E38" t="n">
-        <v>8.5</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7656,16 +7656,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>6.8</v>
+        <v>4.1</v>
       </c>
       <c r="E39" t="n">
-        <v>7.4</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7679,16 +7679,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>6.7</v>
       </c>
       <c r="E40" t="n">
-        <v>5.4</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7702,16 +7702,16 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>21.9</v>
+        <v>21.5</v>
       </c>
       <c r="E41" t="n">
-        <v>29.8</v>
+        <v>26.4</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7725,16 +7725,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>22.9</v>
+        <v>20</v>
       </c>
       <c r="E42" t="n">
-        <v>31.6</v>
+        <v>25.9</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7748,16 +7748,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>6292.1</v>
+        <v>6142.4</v>
       </c>
       <c r="E43" t="n">
-        <v>2835.2</v>
+        <v>2709.1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7771,16 +7771,16 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>99.40000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="E44" t="n">
-        <v>97.3</v>
+        <v>81.3</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7794,16 +7794,16 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1248.9</v>
+        <v>1232.3</v>
       </c>
       <c r="E45" t="n">
-        <v>1035.2</v>
+        <v>978.7</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7817,16 +7817,16 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>10.2</v>
+        <v>1.5</v>
       </c>
       <c r="E46" t="n">
-        <v>13.1</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7840,16 +7840,16 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>10.5</v>
+        <v>2.2</v>
       </c>
       <c r="E47" t="n">
-        <v>16.4</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7863,16 +7863,16 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>23.3</v>
+        <v>21.9</v>
       </c>
       <c r="E48" t="n">
-        <v>33.5</v>
+        <v>27.4</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7886,16 +7886,16 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>49.7</v>
+        <v>40.2</v>
       </c>
       <c r="E49" t="n">
-        <v>58.8</v>
+        <v>46.9</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7909,16 +7909,16 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>44.2</v>
+        <v>34.4</v>
       </c>
       <c r="E50" t="n">
-        <v>59.1</v>
+        <v>45.8</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -7932,16 +7932,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>14.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E51" t="n">
-        <v>14</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -7955,16 +7955,16 @@
         </is>
       </c>
       <c r="D52" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E52" t="n">
         <v>5.1</v>
-      </c>
-      <c r="E52" t="n">
-        <v>6.3</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -7978,16 +7978,16 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-4.9</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="E53" t="n">
-        <v>-2.5</v>
+        <v>-5.9</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -8001,16 +8001,16 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>54.6</v>
+        <v>49.3</v>
       </c>
       <c r="E54" t="n">
-        <v>57.1</v>
+        <v>51.7</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -8024,16 +8024,16 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>12.9</v>
+        <v>10.3</v>
       </c>
       <c r="E55" t="n">
-        <v>16.5</v>
+        <v>13.9</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -8047,13 +8047,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>9.800000000000001</v>
+        <v>3</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -8067,13 +8067,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>8.5</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -8087,13 +8087,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>22.2</v>
+        <v>23.2</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -8107,13 +8107,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>40.3</v>
+        <v>40.1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -8127,13 +8127,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>24.5</v>
+        <v>24.8</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -8156,7 +8156,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -8170,7 +8170,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>10.6</v>
+        <v>10.5</v>
       </c>
       <c r="E62" t="n">
         <v>10</v>
@@ -8179,7 +8179,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -8196,13 +8196,13 @@
         <v>22.8</v>
       </c>
       <c r="E63" t="n">
-        <v>21.3</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -8216,16 +8216,16 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>50</v>
+        <v>49.8</v>
       </c>
       <c r="E64" t="n">
-        <v>47</v>
+        <v>46.9</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -8239,16 +8239,16 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>29.9</v>
+        <v>30.9</v>
       </c>
       <c r="E65" t="n">
-        <v>28.1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -8262,7 +8262,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>2.2</v>
+        <v>1.6</v>
       </c>
       <c r="E66" t="n">
         <v>0.2</v>
@@ -8271,7 +8271,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -8285,7 +8285,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>7.1</v>
+        <v>6.2</v>
       </c>
       <c r="E67" t="n">
         <v>0.6</v>
@@ -8294,7 +8294,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -8308,7 +8308,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>9.6</v>
+        <v>10.4</v>
       </c>
       <c r="E68" t="n">
         <v>1.2</v>
@@ -8317,7 +8317,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -8331,7 +8331,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>22.4</v>
+        <v>22.3</v>
       </c>
       <c r="E69" t="n">
         <v>2.1</v>
@@ -8340,7 +8340,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -8354,16 +8354,16 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>13.7</v>
+        <v>13.9</v>
       </c>
       <c r="E70" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -8377,13 +8377,13 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -8403,7 +8403,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -8417,7 +8417,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
     </row>
   </sheetData>
@@ -8480,7 +8480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8505,7 +8505,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8524,13 +8524,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5.4</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8549,13 +8549,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>9.800000000000001</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8580,7 +8580,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8599,13 +8599,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>12.2</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8630,7 +8630,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8655,7 +8655,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8674,13 +8674,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>21.3</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8699,13 +8699,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>47</v>
+        <v>46.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -8724,13 +8724,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>28.1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -8749,13 +8749,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>3.1</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -8774,13 +8774,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>8.1</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -8799,13 +8799,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>8.199999999999999</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -8824,13 +8824,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>35.7</v>
+        <v>42.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -8849,13 +8849,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>31.8</v>
+        <v>37.2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -8874,13 +8874,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>-6.5</v>
+        <v>-6.1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -8899,13 +8899,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.9</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -8924,13 +8924,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>8.9</v>
+        <v>13.9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -8949,13 +8949,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>33.1</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -8974,13 +8974,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>31.4</v>
+        <v>26.3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -8999,13 +8999,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>14.2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9024,13 +9024,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>11.7</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9049,13 +9049,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>30.7</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9074,13 +9074,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>41.1</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9099,13 +9099,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>30.5</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -9124,13 +9124,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>-9.1</v>
+        <v>-26.1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -9149,13 +9149,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>12.2</v>
+        <v>-7.9</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -9174,13 +9174,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>61.1</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -9199,13 +9199,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>67.8</v>
+        <v>46.2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -9224,13 +9224,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>87.90000000000001</v>
+        <v>63.4</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -9249,13 +9249,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>3.43</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -9274,13 +9274,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>11.13</v>
+        <v>10.74</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -9299,13 +9299,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>22.56</v>
+        <v>22.6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -9324,13 +9324,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>50.12</v>
+        <v>50.02</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -9349,7 +9349,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>30.18</v>
+        <v>31.18</v>
       </c>
     </row>
   </sheetData>
@@ -9497,7 +9497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9511,13 +9511,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>10.21</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9531,13 +9531,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>9.67</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9551,13 +9551,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.43</v>
+        <v>3.14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9571,13 +9571,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5.32</v>
+        <v>4.87</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9591,13 +9591,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.47</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9611,13 +9611,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.78</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9631,13 +9631,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2.74</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9651,13 +9651,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.42</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -9671,13 +9671,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>36.57</v>
+        <v>40.42</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -9691,13 +9691,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3.56</v>
+        <v>2.68</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -9711,13 +9711,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>25.78</v>
+        <v>25.74</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -9731,13 +9731,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -9751,13 +9751,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.37</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -9771,13 +9771,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>69.31999999999999</v>
+        <v>66.98</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -9791,13 +9791,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>30.31</v>
+        <v>29.37</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9811,13 +9811,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>86.81999999999999</v>
+        <v>89.02</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -9831,13 +9831,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>9.65</v>
+        <v>7.35</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -9851,13 +9851,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3.53</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9871,13 +9871,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>10.39</v>
+        <v>10.56</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9891,13 +9891,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>3.19</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9911,13 +9911,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>55.21</v>
+        <v>56.7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9931,13 +9931,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>22.85</v>
+        <v>21.45</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9951,13 +9951,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8.359999999999999</v>
+        <v>8.050000000000001</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9971,13 +9971,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>90.59</v>
+        <v>90.61</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9991,13 +9991,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>7.39</v>
+        <v>7.42</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -10011,13 +10011,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2.02</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -10031,13 +10031,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>88.25</v>
+        <v>89.22</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -10057,7 +10057,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -10067,37 +10067,37 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>10.79</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DGH</t>
+          <t>AYA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1.02</v>
+        <v>9.73</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -10107,17 +10107,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Katılma Hesabı (TL)</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>6.28</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -10127,17 +10127,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.8</v>
+        <v>7.26</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -10147,17 +10147,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>21.58</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -10167,17 +10167,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1.02</v>
+        <v>21.87</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -10187,37 +10187,37 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>69.3</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>JET</t>
+          <t>DGH</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>23.47</v>
+        <v>67.92</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -10227,17 +10227,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>3.66</v>
+        <v>23.19</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -10251,13 +10251,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.14</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -10271,13 +10271,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>66.66</v>
+        <v>70.39</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -10291,13 +10291,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>6.07</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -10317,7 +10317,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -10331,13 +10331,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3.27</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -10351,13 +10351,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>80.09</v>
+        <v>82.42</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -10371,13 +10371,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>7.84</v>
+        <v>5.38</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10391,13 +10391,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>81.68000000000001</v>
+        <v>83.11</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -10411,13 +10411,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>18.32</v>
+        <v>16.89</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -10431,13 +10431,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>21.11</v>
+        <v>19.67</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -10451,13 +10451,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.35</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -10471,13 +10471,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>65.97</v>
+        <v>67.59</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -10491,13 +10491,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>12.57</v>
+        <v>12.55</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -10511,13 +10511,13 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>87.91</v>
+        <v>89.43000000000001</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -10531,13 +10531,13 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>12.09</v>
+        <v>10.57</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10551,13 +10551,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1.46</v>
+        <v>1.54</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -10571,13 +10571,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>16.71</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -10591,13 +10591,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>3.74</v>
+        <v>3.32</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -10617,7 +10617,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -10631,13 +10631,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>67.43000000000001</v>
+        <v>69.59999999999999</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -10651,13 +10651,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>10.64</v>
+        <v>9.42</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -10671,13 +10671,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>31.08</v>
+        <v>28.81</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -10691,13 +10691,13 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.51</v>
+        <v>4.82</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -10711,13 +10711,13 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>67.87</v>
+        <v>65.86</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -10731,7 +10731,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.54</v>
+        <v>0.51</v>
       </c>
     </row>
   </sheetData>
@@ -10841,25 +10841,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>21.9</v>
+        <v>21.5</v>
       </c>
       <c r="E2" t="n">
-        <v>99.40000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>1248.9</v>
+        <v>1232.3</v>
       </c>
       <c r="G2" t="n">
-        <v>6292.1</v>
+        <v>6142.4</v>
       </c>
       <c r="H2" t="n">
-        <v>25.9</v>
+        <v>22.4</v>
       </c>
       <c r="I2" t="n">
-        <v>68.3</v>
+        <v>67.8</v>
       </c>
       <c r="J2" t="n">
-        <v>35.2</v>
+        <v>34.9</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -10884,25 +10884,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>29.8</v>
+        <v>26.4</v>
       </c>
       <c r="E3" t="n">
-        <v>97.3</v>
+        <v>81.3</v>
       </c>
       <c r="F3" t="n">
-        <v>1035.2</v>
+        <v>978.7</v>
       </c>
       <c r="G3" t="n">
-        <v>2835.2</v>
+        <v>2709.1</v>
       </c>
       <c r="H3" t="n">
-        <v>25.4</v>
+        <v>21.9</v>
       </c>
       <c r="I3" t="n">
-        <v>62.6</v>
+        <v>60.9</v>
       </c>
       <c r="J3" t="n">
-        <v>27.8</v>
+        <v>27.3</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -10927,25 +10927,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-7.9</v>
+        <v>-4.9</v>
       </c>
       <c r="E4" t="n">
         <v>2.1</v>
       </c>
       <c r="F4" t="n">
-        <v>213.7</v>
+        <v>253.6</v>
       </c>
       <c r="G4" t="n">
-        <v>3456.9</v>
+        <v>3433.3</v>
       </c>
       <c r="H4" t="n">
         <v>0.5</v>
       </c>
       <c r="I4" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="J4" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -10970,25 +10970,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>24.6</v>
+        <v>24.2</v>
       </c>
       <c r="E5" t="n">
-        <v>110.7</v>
+        <v>93.8</v>
       </c>
       <c r="F5" t="n">
-        <v>1379.4</v>
+        <v>1361.2</v>
       </c>
       <c r="G5" t="n">
-        <v>8020.4</v>
+        <v>7830.2</v>
       </c>
       <c r="H5" t="n">
-        <v>28.2</v>
+        <v>24.7</v>
       </c>
       <c r="I5" t="n">
-        <v>71.40000000000001</v>
+        <v>71</v>
       </c>
       <c r="J5" t="n">
-        <v>37.6</v>
+        <v>37.3</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -11013,25 +11013,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>29.8</v>
+        <v>26.4</v>
       </c>
       <c r="E6" t="n">
-        <v>97.3</v>
+        <v>81.3</v>
       </c>
       <c r="F6" t="n">
-        <v>1035.2</v>
+        <v>978.7</v>
       </c>
       <c r="G6" t="n">
-        <v>2835.2</v>
+        <v>2709.1</v>
       </c>
       <c r="H6" t="n">
-        <v>25.4</v>
+        <v>21.9</v>
       </c>
       <c r="I6" t="n">
-        <v>62.6</v>
+        <v>60.9</v>
       </c>
       <c r="J6" t="n">
-        <v>27.8</v>
+        <v>27.3</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -11056,25 +11056,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-5.2</v>
+        <v>-2.2</v>
       </c>
       <c r="E7" t="n">
-        <v>13.4</v>
+        <v>12.5</v>
       </c>
       <c r="F7" t="n">
-        <v>344.2</v>
+        <v>382.5</v>
       </c>
       <c r="G7" t="n">
-        <v>5185.2</v>
+        <v>5121.1</v>
       </c>
       <c r="H7" t="n">
         <v>2.8</v>
       </c>
       <c r="I7" t="n">
-        <v>8.800000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="J7" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -11148,10 +11148,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>25.9</v>
+        <v>22.4</v>
       </c>
       <c r="E2" t="n">
-        <v>25.4</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="3">
@@ -11171,10 +11171,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3.3</v>
+        <v>0.6</v>
       </c>
       <c r="E3" t="n">
-        <v>2.9</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="4">
@@ -11194,10 +11194,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>68.3</v>
+        <v>67.8</v>
       </c>
       <c r="E4" t="n">
-        <v>62.6</v>
+        <v>60.9</v>
       </c>
     </row>
     <row r="5">
@@ -11217,10 +11217,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>18.6</v>
+        <v>18</v>
       </c>
       <c r="E5" t="n">
-        <v>14.6</v>
+        <v>13.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>